<commit_message>
Noe COD IMS and COD SAP is processing fine
</commit_message>
<xml_diff>
--- a/Viajante/Template.xlsx
+++ b/Viajante/Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="35">
   <si>
     <t>COD FORNECEDOR</t>
   </si>
@@ -43,61 +43,46 @@
     <t>800006503</t>
   </si>
   <si>
+    <t>70690</t>
+  </si>
+  <si>
     <t>1080</t>
   </si>
   <si>
-    <t>463488160</t>
+    <t>1002167600</t>
   </si>
   <si>
-    <t>463554420</t>
+    <t>1002167640</t>
   </si>
   <si>
-    <t>463587560</t>
+    <t>518359540</t>
   </si>
   <si>
-    <t>520420570</t>
+    <t>518442450</t>
   </si>
   <si>
-    <t>520420580</t>
+    <t>519499900</t>
   </si>
   <si>
-    <t>520445670</t>
+    <t>520404360</t>
   </si>
   <si>
-    <t>520542260</t>
+    <t>521286840</t>
   </si>
   <si>
-    <t>521095800</t>
+    <t>521286850</t>
   </si>
   <si>
-    <t>521582000</t>
+    <t>521286870</t>
   </si>
   <si>
-    <t>522310060</t>
+    <t>521286880</t>
   </si>
   <si>
-    <t>522315940</t>
+    <t>521427120</t>
   </si>
   <si>
-    <t>522315950</t>
-  </si>
-  <si>
-    <t>522370320</t>
-  </si>
-  <si>
-    <t>520337470</t>
-  </si>
-  <si>
-    <t>9872247780</t>
-  </si>
-  <si>
-    <t>9874623580</t>
-  </si>
-  <si>
-    <t>9872205180</t>
-  </si>
-  <si>
-    <t>9872255180</t>
+    <t>521491000</t>
   </si>
   <si>
     <t>Apr</t>
@@ -491,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -524,3700 +509,3059 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2">
-        <v>16016</v>
+        <v>2554</v>
       </c>
       <c r="F2">
         <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>8</v>
       </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3">
-        <v>331</v>
+        <v>2554</v>
       </c>
       <c r="F3">
         <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>8</v>
       </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4">
-        <v>18228</v>
+        <v>5107</v>
       </c>
       <c r="F4">
         <v>19</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>8</v>
       </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5">
-        <v>10514</v>
+        <v>2554</v>
       </c>
       <c r="F5">
         <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>8</v>
       </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E6">
-        <v>23067</v>
+        <v>2554</v>
       </c>
       <c r="F6">
         <v>19</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>8</v>
       </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7">
-        <v>11383</v>
+        <v>2554</v>
       </c>
       <c r="F7">
         <v>19</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>8</v>
       </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E8">
-        <v>7779</v>
+        <v>6514</v>
       </c>
       <c r="F8">
         <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E9">
-        <v>11088</v>
+        <v>8460</v>
       </c>
       <c r="F9">
         <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>8</v>
       </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
       <c r="C10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10">
-        <v>8074</v>
+        <v>6514</v>
       </c>
       <c r="F10">
         <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>8</v>
       </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
       <c r="C11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E11">
-        <v>10514</v>
+        <v>8460</v>
       </c>
       <c r="F11">
         <v>19</v>
       </c>
       <c r="H11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>8</v>
       </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12">
-        <v>411</v>
+        <v>14974</v>
       </c>
       <c r="F12">
         <v>19</v>
       </c>
       <c r="H12" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>8</v>
       </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E13">
-        <v>23067</v>
+        <v>4049</v>
       </c>
       <c r="F13">
         <v>19</v>
       </c>
       <c r="H13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>8</v>
       </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
       <c r="C14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E14">
-        <v>3183</v>
+        <v>4049</v>
       </c>
       <c r="F14">
         <v>19</v>
       </c>
       <c r="H14" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>8</v>
       </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
       <c r="C15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E15">
-        <v>22424</v>
+        <v>8098</v>
       </c>
       <c r="F15">
         <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>8</v>
       </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
       <c r="C16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E16">
-        <v>330</v>
+        <v>4049</v>
       </c>
       <c r="F16">
         <v>19</v>
       </c>
       <c r="H16" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>8</v>
       </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
       <c r="C17" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E17">
-        <v>28470</v>
+        <v>4049</v>
       </c>
       <c r="F17">
         <v>19</v>
       </c>
       <c r="H17" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>8</v>
       </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
       <c r="C18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D18" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E18">
-        <v>550</v>
+        <v>4049</v>
       </c>
       <c r="F18">
         <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
         <v>8</v>
       </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
       <c r="C19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D19" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E19">
-        <v>17317</v>
+        <v>9738</v>
       </c>
       <c r="F19">
         <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>8</v>
       </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
       <c r="C20" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D20" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E20">
-        <v>36973</v>
+        <v>14737</v>
       </c>
       <c r="F20">
         <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
         <v>8</v>
       </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
       <c r="C21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D21" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E21">
-        <v>16847</v>
+        <v>9738</v>
       </c>
       <c r="F21">
         <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
         <v>8</v>
       </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
       <c r="C22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D22" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E22">
-        <v>12672</v>
+        <v>14737</v>
       </c>
       <c r="F22">
         <v>19</v>
       </c>
       <c r="H22" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
         <v>8</v>
       </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
       <c r="C23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E23">
-        <v>15049</v>
+        <v>24475</v>
       </c>
       <c r="F23">
         <v>19</v>
       </c>
       <c r="H23" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
         <v>8</v>
       </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
       <c r="C24" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E24">
-        <v>14470</v>
+        <v>2639</v>
       </c>
       <c r="F24">
         <v>19</v>
       </c>
       <c r="H24" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
         <v>8</v>
       </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
       <c r="C25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E25">
-        <v>16767</v>
+        <v>2639</v>
       </c>
       <c r="F25">
         <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
         <v>8</v>
       </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
       <c r="C26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E26">
-        <v>138</v>
+        <v>5278</v>
       </c>
       <c r="F26">
         <v>19</v>
       </c>
       <c r="H26" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
         <v>8</v>
       </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
       <c r="C27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E27">
-        <v>36973</v>
+        <v>2639</v>
       </c>
       <c r="F27">
         <v>19</v>
       </c>
       <c r="H27" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
         <v>8</v>
       </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
       <c r="C28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E28">
-        <v>3600</v>
+        <v>2639</v>
       </c>
       <c r="F28">
         <v>19</v>
       </c>
       <c r="H28" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
         <v>8</v>
       </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E29">
-        <v>1476</v>
+        <v>2639</v>
       </c>
       <c r="F29">
         <v>19</v>
       </c>
       <c r="H29" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
         <v>8</v>
       </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
       <c r="C30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30">
+        <v>8250</v>
+      </c>
+      <c r="F30">
+        <v>19</v>
+      </c>
+      <c r="H30" t="s">
         <v>25</v>
-      </c>
-      <c r="E30">
-        <v>1476</v>
-      </c>
-      <c r="F30">
-        <v>19</v>
-      </c>
-      <c r="H30" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
         <v>8</v>
       </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
       <c r="C31" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D31" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E31">
-        <v>15068</v>
+        <v>7444</v>
       </c>
       <c r="F31">
         <v>19</v>
       </c>
       <c r="H31" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
         <v>8</v>
       </c>
+      <c r="B32" t="s">
+        <v>9</v>
+      </c>
       <c r="C32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D32" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E32">
-        <v>95</v>
+        <v>8250</v>
       </c>
       <c r="F32">
         <v>19</v>
       </c>
       <c r="H32" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
         <v>8</v>
       </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
       <c r="C33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E33">
-        <v>18919</v>
+        <v>7444</v>
       </c>
       <c r="F33">
         <v>19</v>
       </c>
       <c r="H33" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
         <v>8</v>
       </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
       <c r="C34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E34">
-        <v>6043</v>
+        <v>15694</v>
       </c>
       <c r="F34">
         <v>19</v>
       </c>
       <c r="H34" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>8</v>
       </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
       <c r="C35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E35">
-        <v>14008</v>
+        <v>2074</v>
       </c>
       <c r="F35">
         <v>19</v>
       </c>
       <c r="H35" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
         <v>8</v>
       </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
       <c r="C36" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D36" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E36">
-        <v>23005</v>
+        <v>2074</v>
       </c>
       <c r="F36">
         <v>19</v>
       </c>
       <c r="H36" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
         <v>8</v>
       </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
       <c r="C37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D37" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E37">
-        <v>3691</v>
+        <v>4148</v>
       </c>
       <c r="F37">
         <v>19</v>
       </c>
       <c r="H37" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
         <v>8</v>
       </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
       <c r="C38" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E38">
-        <v>8829</v>
+        <v>2074</v>
       </c>
       <c r="F38">
         <v>19</v>
       </c>
       <c r="H38" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
         <v>8</v>
       </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
       <c r="C39" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>2864</v>
+        <v>2074</v>
       </c>
       <c r="F39">
         <v>19</v>
       </c>
       <c r="H39" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
         <v>8</v>
       </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
       <c r="C40" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D40" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>9656</v>
+        <v>2074</v>
       </c>
       <c r="F40">
         <v>19</v>
       </c>
       <c r="H40" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
         <v>8</v>
       </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
       <c r="C41" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E41">
-        <v>7965</v>
+        <v>5186</v>
       </c>
       <c r="F41">
         <v>19</v>
       </c>
       <c r="H41" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
         <v>8</v>
       </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
       <c r="C42" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E42">
-        <v>23005</v>
+        <v>7155</v>
       </c>
       <c r="F42">
         <v>19</v>
       </c>
       <c r="H42" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
         <v>8</v>
       </c>
+      <c r="B43" t="s">
+        <v>9</v>
+      </c>
       <c r="C43" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E43">
-        <v>107</v>
+        <v>5186</v>
       </c>
       <c r="F43">
         <v>19</v>
       </c>
       <c r="H43" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
         <v>8</v>
       </c>
+      <c r="B44" t="s">
+        <v>9</v>
+      </c>
       <c r="C44" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D44" t="s">
+        <v>20</v>
+      </c>
+      <c r="E44">
+        <v>7155</v>
+      </c>
+      <c r="F44">
+        <v>19</v>
+      </c>
+      <c r="H44" t="s">
         <v>26</v>
-      </c>
-      <c r="E44">
-        <v>300</v>
-      </c>
-      <c r="F44">
-        <v>19</v>
-      </c>
-      <c r="H44" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
         <v>8</v>
       </c>
+      <c r="B45" t="s">
+        <v>9</v>
+      </c>
       <c r="C45" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D45" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E45">
-        <v>7358</v>
+        <v>12341</v>
       </c>
       <c r="F45">
         <v>19</v>
       </c>
       <c r="H45" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
         <v>8</v>
       </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
       <c r="C46" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E46">
-        <v>300</v>
+        <v>623</v>
       </c>
       <c r="F46">
         <v>19</v>
       </c>
       <c r="H46" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
         <v>8</v>
       </c>
+      <c r="B47" t="s">
+        <v>9</v>
+      </c>
       <c r="C47" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D47" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="E47">
-        <v>7358</v>
+        <v>3157</v>
       </c>
       <c r="F47">
         <v>19</v>
       </c>
       <c r="H47" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
         <v>8</v>
       </c>
+      <c r="B48" t="s">
+        <v>9</v>
+      </c>
       <c r="C48" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D48" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E48">
-        <v>14082</v>
+        <v>3157</v>
       </c>
       <c r="F48">
         <v>19</v>
       </c>
       <c r="H48" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
         <v>8</v>
       </c>
+      <c r="B49" t="s">
+        <v>9</v>
+      </c>
       <c r="C49" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D49" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E49">
-        <v>316</v>
+        <v>6314</v>
       </c>
       <c r="F49">
         <v>19</v>
       </c>
       <c r="H49" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
         <v>8</v>
       </c>
+      <c r="B50" t="s">
+        <v>9</v>
+      </c>
       <c r="C50" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E50">
-        <v>15639</v>
+        <v>3157</v>
       </c>
       <c r="F50">
         <v>19</v>
       </c>
       <c r="H50" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
         <v>8</v>
       </c>
+      <c r="B51" t="s">
+        <v>9</v>
+      </c>
       <c r="C51" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E51">
-        <v>9136</v>
+        <v>3157</v>
       </c>
       <c r="F51">
         <v>19</v>
       </c>
       <c r="H51" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
         <v>8</v>
       </c>
+      <c r="B52" t="s">
+        <v>9</v>
+      </c>
       <c r="C52" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D52" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19144</v>
+        <v>3157</v>
       </c>
       <c r="F52">
         <v>19</v>
       </c>
       <c r="H52" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
         <v>8</v>
       </c>
+      <c r="B53" t="s">
+        <v>9</v>
+      </c>
       <c r="C53" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D53" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E53">
-        <v>9832</v>
+        <v>7888</v>
       </c>
       <c r="F53">
         <v>19</v>
       </c>
       <c r="H53" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
         <v>8</v>
       </c>
+      <c r="B54" t="s">
+        <v>9</v>
+      </c>
       <c r="C54" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E54">
-        <v>6477</v>
+        <v>10540</v>
       </c>
       <c r="F54">
         <v>19</v>
       </c>
       <c r="H54" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
         <v>8</v>
       </c>
+      <c r="B55" t="s">
+        <v>9</v>
+      </c>
       <c r="C55" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D55" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E55">
-        <v>8950</v>
+        <v>7888</v>
       </c>
       <c r="F55">
         <v>19</v>
       </c>
       <c r="H55" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
         <v>8</v>
       </c>
+      <c r="B56" t="s">
+        <v>9</v>
+      </c>
       <c r="C56" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D56" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E56">
-        <v>7359</v>
+        <v>10540</v>
       </c>
       <c r="F56">
         <v>19</v>
       </c>
       <c r="H56" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
         <v>8</v>
       </c>
+      <c r="B57" t="s">
+        <v>9</v>
+      </c>
       <c r="C57" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E57">
-        <v>9136</v>
+        <v>18428</v>
       </c>
       <c r="F57">
         <v>19</v>
       </c>
       <c r="H57" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
         <v>8</v>
       </c>
+      <c r="B58" t="s">
+        <v>9</v>
+      </c>
       <c r="C58" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D58" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E58">
-        <v>11</v>
+        <v>2960</v>
       </c>
       <c r="F58">
         <v>19</v>
       </c>
       <c r="H58" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
         <v>8</v>
       </c>
+      <c r="B59" t="s">
+        <v>9</v>
+      </c>
       <c r="C59" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D59" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E59">
-        <v>19144</v>
+        <v>2960</v>
       </c>
       <c r="F59">
         <v>19</v>
       </c>
       <c r="H59" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
         <v>8</v>
       </c>
+      <c r="B60" t="s">
+        <v>9</v>
+      </c>
       <c r="C60" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E60">
-        <v>1754</v>
+        <v>5920</v>
       </c>
       <c r="F60">
         <v>19</v>
       </c>
       <c r="H60" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
         <v>8</v>
       </c>
+      <c r="B61" t="s">
+        <v>9</v>
+      </c>
       <c r="C61" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D61" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E61">
-        <v>42</v>
+        <v>2960</v>
       </c>
       <c r="F61">
         <v>19</v>
       </c>
       <c r="H61" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
         <v>8</v>
       </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
       <c r="C62" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E62">
-        <v>42</v>
+        <v>2960</v>
       </c>
       <c r="F62">
         <v>19</v>
       </c>
       <c r="H62" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
         <v>8</v>
       </c>
+      <c r="B63" t="s">
+        <v>9</v>
+      </c>
       <c r="C63" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D63" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E63">
-        <v>16606</v>
+        <v>2960</v>
       </c>
       <c r="F63">
         <v>19</v>
       </c>
       <c r="H63" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
         <v>8</v>
       </c>
+      <c r="B64" t="s">
+        <v>9</v>
+      </c>
       <c r="C64" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D64" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E64">
-        <v>295</v>
+        <v>6186</v>
       </c>
       <c r="F64">
         <v>19</v>
       </c>
       <c r="H64" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
         <v>8</v>
       </c>
+      <c r="B65" t="s">
+        <v>9</v>
+      </c>
       <c r="C65" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D65" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E65">
-        <v>24461</v>
+        <v>10704</v>
       </c>
       <c r="F65">
         <v>19</v>
       </c>
       <c r="H65" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
         <v>8</v>
       </c>
+      <c r="B66" t="s">
+        <v>9</v>
+      </c>
       <c r="C66" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D66" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E66">
-        <v>7129</v>
+        <v>6186</v>
       </c>
       <c r="F66">
         <v>19</v>
       </c>
       <c r="H66" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
         <v>8</v>
       </c>
+      <c r="B67" t="s">
+        <v>9</v>
+      </c>
       <c r="C67" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D67" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E67">
-        <v>17007</v>
+        <v>10704</v>
       </c>
       <c r="F67">
         <v>19</v>
       </c>
       <c r="H67" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
         <v>8</v>
       </c>
+      <c r="B68" t="s">
+        <v>9</v>
+      </c>
       <c r="C68" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D68" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E68">
-        <v>21391</v>
+        <v>16890</v>
       </c>
       <c r="F68">
         <v>19</v>
       </c>
       <c r="H68" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
         <v>8</v>
       </c>
+      <c r="B69" t="s">
+        <v>9</v>
+      </c>
       <c r="C69" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D69" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E69">
-        <v>4604</v>
+        <v>2705</v>
       </c>
       <c r="F69">
         <v>19</v>
       </c>
       <c r="H69" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
         <v>8</v>
       </c>
+      <c r="B70" t="s">
+        <v>9</v>
+      </c>
       <c r="C70" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E70">
-        <v>7355</v>
+        <v>2705</v>
       </c>
       <c r="F70">
         <v>19</v>
       </c>
       <c r="H70" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
         <v>8</v>
       </c>
+      <c r="B71" t="s">
+        <v>9</v>
+      </c>
       <c r="C71" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E71">
-        <v>11959</v>
+        <v>5410</v>
       </c>
       <c r="F71">
         <v>19</v>
       </c>
       <c r="H71" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
         <v>8</v>
       </c>
+      <c r="B72" t="s">
+        <v>9</v>
+      </c>
       <c r="C72" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E72">
-        <v>9878</v>
+        <v>2705</v>
       </c>
       <c r="F72">
         <v>19</v>
       </c>
       <c r="H72" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
         <v>8</v>
       </c>
+      <c r="B73" t="s">
+        <v>9</v>
+      </c>
       <c r="C73" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D73" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E73">
-        <v>21391</v>
+        <v>2705</v>
       </c>
       <c r="F73">
         <v>19</v>
       </c>
       <c r="H73" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
         <v>8</v>
       </c>
+      <c r="B74" t="s">
+        <v>9</v>
+      </c>
       <c r="C74" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D74" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E74">
-        <v>3016</v>
+        <v>2705</v>
       </c>
       <c r="F74">
         <v>19</v>
       </c>
       <c r="H74" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
         <v>8</v>
       </c>
+      <c r="B75" t="s">
+        <v>9</v>
+      </c>
       <c r="C75" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D75" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E75">
-        <v>300</v>
+        <v>7728</v>
       </c>
       <c r="F75">
         <v>19</v>
       </c>
       <c r="H75" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
         <v>8</v>
       </c>
+      <c r="B76" t="s">
+        <v>9</v>
+      </c>
       <c r="C76" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D76" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E76">
-        <v>8685</v>
+        <v>7823</v>
       </c>
       <c r="F76">
         <v>19</v>
       </c>
       <c r="H76" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
         <v>8</v>
       </c>
+      <c r="B77" t="s">
+        <v>9</v>
+      </c>
       <c r="C77" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D77" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E77">
-        <v>300</v>
+        <v>7728</v>
       </c>
       <c r="F77">
         <v>19</v>
       </c>
       <c r="H77" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
         <v>8</v>
       </c>
+      <c r="B78" t="s">
+        <v>9</v>
+      </c>
       <c r="C78" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D78" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E78">
-        <v>8685</v>
+        <v>7823</v>
       </c>
       <c r="F78">
         <v>19</v>
       </c>
       <c r="H78" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
         <v>8</v>
       </c>
+      <c r="B79" t="s">
+        <v>9</v>
+      </c>
       <c r="C79" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D79" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E79">
-        <v>18433</v>
+        <v>15551</v>
       </c>
       <c r="F79">
         <v>19</v>
       </c>
       <c r="H79" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
         <v>8</v>
       </c>
+      <c r="B80" t="s">
+        <v>9</v>
+      </c>
       <c r="C80" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D80" t="s">
         <v>11</v>
       </c>
       <c r="E80">
-        <v>327</v>
+        <v>3735</v>
       </c>
       <c r="F80">
         <v>19</v>
       </c>
       <c r="H80" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
         <v>8</v>
       </c>
+      <c r="B81" t="s">
+        <v>9</v>
+      </c>
       <c r="C81" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D81" t="s">
         <v>12</v>
       </c>
       <c r="E81">
-        <v>23016</v>
+        <v>3735</v>
       </c>
       <c r="F81">
         <v>19</v>
       </c>
       <c r="H81" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
         <v>8</v>
       </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
       <c r="C82" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D82" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E82">
-        <v>151</v>
+        <v>7470</v>
       </c>
       <c r="F82">
         <v>19</v>
       </c>
       <c r="H82" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
         <v>8</v>
       </c>
+      <c r="B83" t="s">
+        <v>9</v>
+      </c>
       <c r="C83" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D83" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E83">
-        <v>10864</v>
+        <v>3735</v>
       </c>
       <c r="F83">
         <v>19</v>
       </c>
       <c r="H83" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
         <v>8</v>
       </c>
+      <c r="B84" t="s">
+        <v>9</v>
+      </c>
       <c r="C84" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D84" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E84">
-        <v>24385</v>
+        <v>3735</v>
       </c>
       <c r="F84">
         <v>19</v>
       </c>
       <c r="H84" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
         <v>8</v>
       </c>
+      <c r="B85" t="s">
+        <v>9</v>
+      </c>
       <c r="C85" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D85" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E85">
-        <v>13190</v>
+        <v>3735</v>
       </c>
       <c r="F85">
         <v>19</v>
       </c>
       <c r="H85" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
         <v>8</v>
       </c>
+      <c r="B86" t="s">
+        <v>9</v>
+      </c>
       <c r="C86" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D86" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E86">
-        <v>8218</v>
+        <v>9405</v>
       </c>
       <c r="F86">
         <v>19</v>
       </c>
       <c r="H86" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
         <v>8</v>
       </c>
+      <c r="B87" t="s">
+        <v>9</v>
+      </c>
       <c r="C87" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D87" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E87">
-        <v>11218</v>
+        <v>11879</v>
       </c>
       <c r="F87">
         <v>19</v>
       </c>
       <c r="H87" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
         <v>8</v>
       </c>
+      <c r="B88" t="s">
+        <v>9</v>
+      </c>
       <c r="C88" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D88" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E88">
-        <v>10190</v>
+        <v>9405</v>
       </c>
       <c r="F88">
         <v>19</v>
       </c>
       <c r="H88" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
         <v>8</v>
       </c>
+      <c r="B89" t="s">
+        <v>9</v>
+      </c>
       <c r="C89" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D89" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E89">
-        <v>10713</v>
+        <v>11879</v>
       </c>
       <c r="F89">
         <v>19</v>
       </c>
       <c r="H89" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
         <v>8</v>
       </c>
+      <c r="B90" t="s">
+        <v>9</v>
+      </c>
       <c r="C90" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D90" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E90">
-        <v>125</v>
+        <v>21284</v>
       </c>
       <c r="F90">
         <v>19</v>
       </c>
       <c r="H90" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
         <v>8</v>
       </c>
+      <c r="B91" t="s">
+        <v>9</v>
+      </c>
       <c r="C91" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D91" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E91">
-        <v>24385</v>
+        <v>3888</v>
       </c>
       <c r="F91">
         <v>19</v>
       </c>
       <c r="H91" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
         <v>8</v>
       </c>
+      <c r="B92" t="s">
+        <v>9</v>
+      </c>
       <c r="C92" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D92" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E92">
-        <v>3717</v>
+        <v>3888</v>
       </c>
       <c r="F92">
         <v>19</v>
       </c>
       <c r="H92" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
         <v>8</v>
       </c>
+      <c r="B93" t="s">
+        <v>9</v>
+      </c>
       <c r="C93" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D93" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E93">
-        <v>276</v>
+        <v>7777</v>
       </c>
       <c r="F93">
         <v>19</v>
       </c>
       <c r="H93" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
         <v>8</v>
       </c>
+      <c r="B94" t="s">
+        <v>9</v>
+      </c>
       <c r="C94" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D94" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E94">
-        <v>276</v>
+        <v>3888</v>
       </c>
       <c r="F94">
         <v>19</v>
       </c>
       <c r="H94" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
         <v>8</v>
       </c>
+      <c r="B95" t="s">
+        <v>9</v>
+      </c>
       <c r="C95" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D95" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E95">
-        <v>16778</v>
+        <v>3888</v>
       </c>
       <c r="F95">
         <v>19</v>
       </c>
       <c r="H95" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
         <v>8</v>
       </c>
+      <c r="B96" t="s">
+        <v>9</v>
+      </c>
       <c r="C96" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D96" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E96">
-        <v>96</v>
+        <v>3888</v>
       </c>
       <c r="F96">
         <v>19</v>
       </c>
       <c r="H96" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
         <v>8</v>
       </c>
+      <c r="B97" t="s">
+        <v>9</v>
+      </c>
       <c r="C97" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D97" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E97">
-        <v>19772</v>
+        <v>9161</v>
       </c>
       <c r="F97">
         <v>19</v>
       </c>
       <c r="H97" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
         <v>8</v>
       </c>
+      <c r="B98" t="s">
+        <v>9</v>
+      </c>
       <c r="C98" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D98" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E98">
-        <v>7</v>
+        <v>12565</v>
       </c>
       <c r="F98">
         <v>19</v>
       </c>
       <c r="H98" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
         <v>8</v>
       </c>
+      <c r="B99" t="s">
+        <v>9</v>
+      </c>
       <c r="C99" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D99" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E99">
-        <v>11575</v>
+        <v>9161</v>
       </c>
       <c r="F99">
         <v>19</v>
       </c>
       <c r="H99" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
         <v>8</v>
       </c>
+      <c r="B100" t="s">
+        <v>9</v>
+      </c>
       <c r="C100" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D100" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E100">
-        <v>25545</v>
+        <v>12565</v>
       </c>
       <c r="F100">
         <v>19</v>
       </c>
       <c r="H100" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
         <v>8</v>
       </c>
+      <c r="B101" t="s">
+        <v>9</v>
+      </c>
       <c r="C101" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D101" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E101">
-        <v>12013</v>
+        <v>21726</v>
       </c>
       <c r="F101">
         <v>19</v>
       </c>
       <c r="H101" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
         <v>8</v>
       </c>
+      <c r="B102" t="s">
+        <v>9</v>
+      </c>
       <c r="C102" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D102" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E102">
-        <v>9285</v>
+        <v>3784</v>
       </c>
       <c r="F102">
         <v>19</v>
       </c>
       <c r="H102" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
         <v>8</v>
       </c>
+      <c r="B103" t="s">
+        <v>9</v>
+      </c>
       <c r="C103" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D103" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E103">
-        <v>12111</v>
+        <v>3784</v>
       </c>
       <c r="F103">
         <v>19</v>
       </c>
       <c r="H103" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
         <v>8</v>
       </c>
+      <c r="B104" t="s">
+        <v>9</v>
+      </c>
       <c r="C104" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D104" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E104">
-        <v>9187</v>
+        <v>7568</v>
       </c>
       <c r="F104">
         <v>19</v>
       </c>
       <c r="H104" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
         <v>8</v>
       </c>
+      <c r="B105" t="s">
+        <v>9</v>
+      </c>
       <c r="C105" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D105" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E105">
-        <v>11568</v>
+        <v>3784</v>
       </c>
       <c r="F105">
         <v>19</v>
       </c>
       <c r="H105" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
         <v>8</v>
       </c>
+      <c r="B106" t="s">
+        <v>9</v>
+      </c>
       <c r="C106" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D106" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E106">
-        <v>121</v>
+        <v>3784</v>
       </c>
       <c r="F106">
         <v>19</v>
       </c>
       <c r="H106" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="107" spans="1:8">
       <c r="A107" t="s">
         <v>8</v>
       </c>
+      <c r="B107" t="s">
+        <v>9</v>
+      </c>
       <c r="C107" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D107" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E107">
-        <v>25545</v>
+        <v>3784</v>
       </c>
       <c r="F107">
         <v>19</v>
       </c>
       <c r="H107" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
         <v>8</v>
       </c>
+      <c r="B108" t="s">
+        <v>9</v>
+      </c>
       <c r="C108" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D108" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E108">
-        <v>1831</v>
+        <v>7869</v>
       </c>
       <c r="F108">
         <v>19</v>
       </c>
       <c r="H108" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
         <v>8</v>
       </c>
+      <c r="B109" t="s">
+        <v>9</v>
+      </c>
       <c r="C109" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D109" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E109">
-        <v>30</v>
+        <v>14381</v>
       </c>
       <c r="F109">
         <v>19</v>
       </c>
       <c r="H109" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="110" spans="1:8">
       <c r="A110" t="s">
         <v>8</v>
       </c>
+      <c r="B110" t="s">
+        <v>9</v>
+      </c>
       <c r="C110" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D110" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E110">
-        <v>30</v>
+        <v>7869</v>
       </c>
       <c r="F110">
         <v>19</v>
       </c>
       <c r="H110" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="111" spans="1:8">
       <c r="A111" t="s">
         <v>8</v>
       </c>
+      <c r="B111" t="s">
+        <v>9</v>
+      </c>
       <c r="C111" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D111" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E111">
-        <v>20272</v>
+        <v>14381</v>
       </c>
       <c r="F111">
         <v>19</v>
       </c>
       <c r="H111" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="112" spans="1:8">
       <c r="A112" t="s">
         <v>8</v>
       </c>
+      <c r="B112" t="s">
+        <v>9</v>
+      </c>
       <c r="C112" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D112" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E112">
-        <v>267</v>
+        <v>22250</v>
       </c>
       <c r="F112">
         <v>19</v>
       </c>
       <c r="H112" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
         <v>8</v>
       </c>
+      <c r="B113" t="s">
+        <v>9</v>
+      </c>
       <c r="C113" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D113" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E113">
-        <v>24924</v>
+        <v>3302</v>
       </c>
       <c r="F113">
         <v>19</v>
       </c>
       <c r="H113" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="114" spans="1:8">
       <c r="A114" t="s">
         <v>8</v>
       </c>
+      <c r="B114" t="s">
+        <v>9</v>
+      </c>
       <c r="C114" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D114" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E114">
-        <v>15572</v>
+        <v>3302</v>
       </c>
       <c r="F114">
         <v>19</v>
       </c>
       <c r="H114" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="115" spans="1:8">
       <c r="A115" t="s">
         <v>8</v>
       </c>
+      <c r="B115" t="s">
+        <v>9</v>
+      </c>
       <c r="C115" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D115" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E115">
-        <v>32977</v>
+        <v>6604</v>
       </c>
       <c r="F115">
         <v>19</v>
       </c>
       <c r="H115" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="116" spans="1:8">
       <c r="A116" t="s">
         <v>8</v>
       </c>
+      <c r="B116" t="s">
+        <v>9</v>
+      </c>
       <c r="C116" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D116" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E116">
-        <v>16099</v>
+        <v>3302</v>
       </c>
       <c r="F116">
         <v>19</v>
       </c>
       <c r="H116" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="117" spans="1:8">
       <c r="A117" t="s">
         <v>8</v>
       </c>
+      <c r="B117" t="s">
+        <v>9</v>
+      </c>
       <c r="C117" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D117" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E117">
-        <v>10916</v>
+        <v>3302</v>
       </c>
       <c r="F117">
         <v>19</v>
       </c>
       <c r="H117" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="118" spans="1:8">
       <c r="A118" t="s">
         <v>8</v>
       </c>
+      <c r="B118" t="s">
+        <v>9</v>
+      </c>
       <c r="C118" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D118" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E118">
-        <v>15010</v>
+        <v>3302</v>
       </c>
       <c r="F118">
         <v>19</v>
       </c>
       <c r="H118" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="119" spans="1:8">
       <c r="A119" t="s">
         <v>8</v>
       </c>
+      <c r="B119" t="s">
+        <v>9</v>
+      </c>
       <c r="C119" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D119" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E119">
-        <v>12005</v>
+        <v>7873</v>
       </c>
       <c r="F119">
         <v>19</v>
       </c>
       <c r="H119" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="120" spans="1:8">
       <c r="A120" t="s">
         <v>8</v>
       </c>
+      <c r="B120" t="s">
+        <v>9</v>
+      </c>
       <c r="C120" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D120" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E120">
-        <v>15572</v>
+        <v>10991</v>
       </c>
       <c r="F120">
         <v>19</v>
       </c>
       <c r="H120" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="121" spans="1:8">
       <c r="A121" t="s">
         <v>8</v>
       </c>
+      <c r="B121" t="s">
+        <v>9</v>
+      </c>
       <c r="C121" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D121" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E121">
-        <v>32977</v>
+        <v>7873</v>
       </c>
       <c r="F121">
         <v>19</v>
       </c>
       <c r="H121" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="122" spans="1:8">
       <c r="A122" t="s">
         <v>8</v>
       </c>
+      <c r="B122" t="s">
+        <v>9</v>
+      </c>
       <c r="C122" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D122" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E122">
-        <v>3132</v>
+        <v>10991</v>
       </c>
       <c r="F122">
         <v>19</v>
       </c>
       <c r="H122" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="123" spans="1:8">
       <c r="A123" t="s">
         <v>8</v>
       </c>
+      <c r="B123" t="s">
+        <v>9</v>
+      </c>
       <c r="C123" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D123" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E123">
-        <v>23264</v>
+        <v>18864</v>
       </c>
       <c r="F123">
         <v>19</v>
       </c>
       <c r="H123" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="124" spans="1:8">
       <c r="A124" t="s">
         <v>8</v>
       </c>
+      <c r="B124" t="s">
+        <v>9</v>
+      </c>
       <c r="C124" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D124" t="s">
         <v>11</v>
       </c>
       <c r="E124">
-        <v>492</v>
+        <v>3212</v>
       </c>
       <c r="F124">
         <v>19</v>
       </c>
       <c r="H124" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:8">
       <c r="A125" t="s">
         <v>8</v>
       </c>
+      <c r="B125" t="s">
+        <v>9</v>
+      </c>
       <c r="C125" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D125" t="s">
         <v>12</v>
       </c>
       <c r="E125">
-        <v>29845</v>
+        <v>3212</v>
       </c>
       <c r="F125">
         <v>19</v>
       </c>
       <c r="H125" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="126" spans="1:8">
       <c r="A126" t="s">
         <v>8</v>
       </c>
+      <c r="B126" t="s">
+        <v>9</v>
+      </c>
       <c r="C126" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D126" t="s">
         <v>13</v>
       </c>
       <c r="E126">
-        <v>17622</v>
+        <v>6424</v>
       </c>
       <c r="F126">
         <v>19</v>
       </c>
       <c r="H126" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:8">
       <c r="A127" t="s">
         <v>8</v>
       </c>
+      <c r="B127" t="s">
+        <v>9</v>
+      </c>
       <c r="C127" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D127" t="s">
         <v>14</v>
       </c>
       <c r="E127">
-        <v>31611</v>
+        <v>3212</v>
       </c>
       <c r="F127">
         <v>19</v>
       </c>
       <c r="H127" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="128" spans="1:8">
       <c r="A128" t="s">
         <v>8</v>
       </c>
+      <c r="B128" t="s">
+        <v>9</v>
+      </c>
       <c r="C128" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D128" t="s">
         <v>15</v>
       </c>
       <c r="E128">
-        <v>16937</v>
+        <v>3212</v>
       </c>
       <c r="F128">
         <v>19</v>
       </c>
       <c r="H128" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="129" spans="1:8">
       <c r="A129" t="s">
         <v>8</v>
       </c>
+      <c r="B129" t="s">
+        <v>9</v>
+      </c>
       <c r="C129" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D129" t="s">
         <v>16</v>
       </c>
       <c r="E129">
-        <v>11586</v>
+        <v>3212</v>
       </c>
       <c r="F129">
         <v>19</v>
       </c>
       <c r="H129" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="130" spans="1:8">
       <c r="A130" t="s">
         <v>8</v>
       </c>
+      <c r="B130" t="s">
+        <v>9</v>
+      </c>
       <c r="C130" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D130" t="s">
         <v>17</v>
       </c>
       <c r="E130">
-        <v>15209</v>
+        <v>10490</v>
       </c>
       <c r="F130">
         <v>19</v>
       </c>
       <c r="H130" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="131" spans="1:8">
       <c r="A131" t="s">
         <v>8</v>
       </c>
+      <c r="B131" t="s">
+        <v>9</v>
+      </c>
       <c r="C131" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D131" t="s">
         <v>18</v>
       </c>
       <c r="E131">
-        <v>13314</v>
+        <v>7637</v>
       </c>
       <c r="F131">
         <v>19</v>
       </c>
       <c r="H131" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="132" spans="1:8">
       <c r="A132" t="s">
         <v>8</v>
       </c>
+      <c r="B132" t="s">
+        <v>9</v>
+      </c>
       <c r="C132" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D132" t="s">
         <v>19</v>
       </c>
       <c r="E132">
-        <v>17622</v>
+        <v>10490</v>
       </c>
       <c r="F132">
         <v>19</v>
       </c>
       <c r="H132" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="133" spans="1:8">
       <c r="A133" t="s">
         <v>8</v>
       </c>
+      <c r="B133" t="s">
+        <v>9</v>
+      </c>
       <c r="C133" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D133" t="s">
         <v>20</v>
       </c>
       <c r="E133">
-        <v>525</v>
+        <v>7637</v>
       </c>
       <c r="F133">
         <v>19</v>
       </c>
       <c r="H133" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="134" spans="1:8">
       <c r="A134" t="s">
         <v>8</v>
       </c>
+      <c r="B134" t="s">
+        <v>9</v>
+      </c>
       <c r="C134" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D134" t="s">
         <v>21</v>
       </c>
       <c r="E134">
-        <v>31611</v>
+        <v>18127</v>
       </c>
       <c r="F134">
         <v>19</v>
       </c>
       <c r="H134" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="135" spans="1:8">
-      <c r="A135" t="s">
-        <v>8</v>
-      </c>
-      <c r="C135" t="s">
-        <v>9</v>
-      </c>
-      <c r="D135" t="s">
-        <v>22</v>
-      </c>
-      <c r="E135">
-        <v>4688</v>
-      </c>
-      <c r="F135">
-        <v>19</v>
-      </c>
-      <c r="H135" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="136" spans="1:8">
-      <c r="A136" t="s">
-        <v>8</v>
-      </c>
-      <c r="C136" t="s">
-        <v>9</v>
-      </c>
-      <c r="D136" t="s">
-        <v>10</v>
-      </c>
-      <c r="E136">
-        <v>21786</v>
-      </c>
-      <c r="F136">
-        <v>19</v>
-      </c>
-      <c r="H136" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8">
-      <c r="A137" t="s">
-        <v>8</v>
-      </c>
-      <c r="C137" t="s">
-        <v>9</v>
-      </c>
-      <c r="D137" t="s">
-        <v>11</v>
-      </c>
-      <c r="E137">
-        <v>555</v>
-      </c>
-      <c r="F137">
-        <v>19</v>
-      </c>
-      <c r="H137" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8">
-      <c r="A138" t="s">
-        <v>8</v>
-      </c>
-      <c r="C138" t="s">
-        <v>9</v>
-      </c>
-      <c r="D138" t="s">
-        <v>12</v>
-      </c>
-      <c r="E138">
-        <v>33114</v>
-      </c>
-      <c r="F138">
-        <v>19</v>
-      </c>
-      <c r="H138" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="139" spans="1:8">
-      <c r="A139" t="s">
-        <v>8</v>
-      </c>
-      <c r="C139" t="s">
-        <v>9</v>
-      </c>
-      <c r="D139" t="s">
-        <v>23</v>
-      </c>
-      <c r="E139">
-        <v>8449</v>
-      </c>
-      <c r="F139">
-        <v>19</v>
-      </c>
-      <c r="H139" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="140" spans="1:8">
-      <c r="A140" t="s">
-        <v>8</v>
-      </c>
-      <c r="C140" t="s">
-        <v>9</v>
-      </c>
-      <c r="D140" t="s">
-        <v>13</v>
-      </c>
-      <c r="E140">
-        <v>20744</v>
-      </c>
-      <c r="F140">
-        <v>19</v>
-      </c>
-      <c r="H140" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="141" spans="1:8">
-      <c r="A141" t="s">
-        <v>8</v>
-      </c>
-      <c r="C141" t="s">
-        <v>9</v>
-      </c>
-      <c r="D141" t="s">
-        <v>14</v>
-      </c>
-      <c r="E141">
-        <v>28147</v>
-      </c>
-      <c r="F141">
-        <v>19</v>
-      </c>
-      <c r="H141" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8">
-      <c r="A142" t="s">
-        <v>8</v>
-      </c>
-      <c r="C142" t="s">
-        <v>9</v>
-      </c>
-      <c r="D142" t="s">
-        <v>15</v>
-      </c>
-      <c r="E142">
-        <v>5205</v>
-      </c>
-      <c r="F142">
-        <v>19</v>
-      </c>
-      <c r="H142" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="143" spans="1:8">
-      <c r="A143" t="s">
-        <v>8</v>
-      </c>
-      <c r="C143" t="s">
-        <v>9</v>
-      </c>
-      <c r="D143" t="s">
-        <v>16</v>
-      </c>
-      <c r="E143">
-        <v>13432</v>
-      </c>
-      <c r="F143">
-        <v>19</v>
-      </c>
-      <c r="H143" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="144" spans="1:8">
-      <c r="A144" t="s">
-        <v>8</v>
-      </c>
-      <c r="C144" t="s">
-        <v>9</v>
-      </c>
-      <c r="D144" t="s">
-        <v>17</v>
-      </c>
-      <c r="E144">
-        <v>4751</v>
-      </c>
-      <c r="F144">
-        <v>19</v>
-      </c>
-      <c r="H144" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="145" spans="1:8">
-      <c r="A145" t="s">
-        <v>8</v>
-      </c>
-      <c r="C145" t="s">
-        <v>9</v>
-      </c>
-      <c r="D145" t="s">
-        <v>18</v>
-      </c>
-      <c r="E145">
-        <v>13886</v>
-      </c>
-      <c r="F145">
-        <v>19</v>
-      </c>
-      <c r="H145" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="146" spans="1:8">
-      <c r="A146" t="s">
-        <v>8</v>
-      </c>
-      <c r="C146" t="s">
-        <v>9</v>
-      </c>
-      <c r="D146" t="s">
-        <v>19</v>
-      </c>
-      <c r="E146">
-        <v>12295</v>
-      </c>
-      <c r="F146">
-        <v>19</v>
-      </c>
-      <c r="H146" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="147" spans="1:8">
-      <c r="A147" t="s">
-        <v>8</v>
-      </c>
-      <c r="C147" t="s">
-        <v>9</v>
-      </c>
-      <c r="D147" t="s">
-        <v>21</v>
-      </c>
-      <c r="E147">
-        <v>28147</v>
-      </c>
-      <c r="F147">
-        <v>19</v>
-      </c>
-      <c r="H147" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8">
-      <c r="A148" t="s">
-        <v>8</v>
-      </c>
-      <c r="C148" t="s">
-        <v>9</v>
-      </c>
-      <c r="D148" t="s">
-        <v>22</v>
-      </c>
-      <c r="E148">
-        <v>5821</v>
-      </c>
-      <c r="F148">
-        <v>19</v>
-      </c>
-      <c r="H148" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="149" spans="1:8">
-      <c r="A149" t="s">
-        <v>8</v>
-      </c>
-      <c r="C149" t="s">
-        <v>9</v>
-      </c>
-      <c r="D149" t="s">
-        <v>26</v>
-      </c>
-      <c r="E149">
-        <v>300</v>
-      </c>
-      <c r="F149">
-        <v>19</v>
-      </c>
-      <c r="H149" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="150" spans="1:8">
-      <c r="A150" t="s">
-        <v>8</v>
-      </c>
-      <c r="C150" t="s">
-        <v>9</v>
-      </c>
-      <c r="D150" t="s">
-        <v>24</v>
-      </c>
-      <c r="E150">
-        <v>10760</v>
-      </c>
-      <c r="F150">
-        <v>19</v>
-      </c>
-      <c r="H150" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8">
-      <c r="A151" t="s">
-        <v>8</v>
-      </c>
-      <c r="C151" t="s">
-        <v>9</v>
-      </c>
-      <c r="D151" t="s">
-        <v>27</v>
-      </c>
-      <c r="E151">
-        <v>300</v>
-      </c>
-      <c r="F151">
-        <v>19</v>
-      </c>
-      <c r="H151" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8">
-      <c r="A152" t="s">
-        <v>8</v>
-      </c>
-      <c r="C152" t="s">
-        <v>9</v>
-      </c>
-      <c r="D152" t="s">
-        <v>25</v>
-      </c>
-      <c r="E152">
-        <v>10760</v>
-      </c>
-      <c r="F152">
-        <v>19</v>
-      </c>
-      <c r="H152" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8">
-      <c r="A153" t="s">
-        <v>8</v>
-      </c>
-      <c r="C153" t="s">
-        <v>9</v>
-      </c>
-      <c r="D153" t="s">
-        <v>10</v>
-      </c>
-      <c r="E153">
-        <v>17433</v>
-      </c>
-      <c r="F153">
-        <v>19</v>
-      </c>
-      <c r="H153" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8">
-      <c r="A154" t="s">
-        <v>8</v>
-      </c>
-      <c r="C154" t="s">
-        <v>9</v>
-      </c>
-      <c r="D154" t="s">
-        <v>11</v>
-      </c>
-      <c r="E154">
-        <v>245</v>
-      </c>
-      <c r="F154">
-        <v>19</v>
-      </c>
-      <c r="H154" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="155" spans="1:8">
-      <c r="A155" t="s">
-        <v>8</v>
-      </c>
-      <c r="C155" t="s">
-        <v>9</v>
-      </c>
-      <c r="D155" t="s">
-        <v>12</v>
-      </c>
-      <c r="E155">
-        <v>25359</v>
-      </c>
-      <c r="F155">
-        <v>19</v>
-      </c>
-      <c r="H155" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8">
-      <c r="A156" t="s">
-        <v>8</v>
-      </c>
-      <c r="C156" t="s">
-        <v>9</v>
-      </c>
-      <c r="D156" t="s">
-        <v>23</v>
-      </c>
-      <c r="E156">
-        <v>4436</v>
-      </c>
-      <c r="F156">
-        <v>19</v>
-      </c>
-      <c r="H156" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8">
-      <c r="A157" t="s">
-        <v>8</v>
-      </c>
-      <c r="C157" t="s">
-        <v>9</v>
-      </c>
-      <c r="D157" t="s">
-        <v>13</v>
-      </c>
-      <c r="E157">
-        <v>17266</v>
-      </c>
-      <c r="F157">
-        <v>19</v>
-      </c>
-      <c r="H157" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="158" spans="1:8">
-      <c r="A158" t="s">
-        <v>8</v>
-      </c>
-      <c r="C158" t="s">
-        <v>9</v>
-      </c>
-      <c r="D158" t="s">
-        <v>14</v>
-      </c>
-      <c r="E158">
-        <v>25604</v>
-      </c>
-      <c r="F158">
-        <v>19</v>
-      </c>
-      <c r="H158" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="159" spans="1:8">
-      <c r="A159" t="s">
-        <v>8</v>
-      </c>
-      <c r="C159" t="s">
-        <v>9</v>
-      </c>
-      <c r="D159" t="s">
-        <v>15</v>
-      </c>
-      <c r="E159">
-        <v>6920</v>
-      </c>
-      <c r="F159">
-        <v>19</v>
-      </c>
-      <c r="H159" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="160" spans="1:8">
-      <c r="A160" t="s">
-        <v>8</v>
-      </c>
-      <c r="C160" t="s">
-        <v>9</v>
-      </c>
-      <c r="D160" t="s">
-        <v>16</v>
-      </c>
-      <c r="E160">
-        <v>10844</v>
-      </c>
-      <c r="F160">
-        <v>19</v>
-      </c>
-      <c r="H160" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="161" spans="1:8">
-      <c r="A161" t="s">
-        <v>8</v>
-      </c>
-      <c r="C161" t="s">
-        <v>9</v>
-      </c>
-      <c r="D161" t="s">
-        <v>17</v>
-      </c>
-      <c r="E161">
-        <v>5932</v>
-      </c>
-      <c r="F161">
-        <v>19</v>
-      </c>
-      <c r="H161" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="162" spans="1:8">
-      <c r="A162" t="s">
-        <v>8</v>
-      </c>
-      <c r="C162" t="s">
-        <v>9</v>
-      </c>
-      <c r="D162" t="s">
-        <v>18</v>
-      </c>
-      <c r="E162">
-        <v>11832</v>
-      </c>
-      <c r="F162">
-        <v>19</v>
-      </c>
-      <c r="H162" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="163" spans="1:8">
-      <c r="A163" t="s">
-        <v>8</v>
-      </c>
-      <c r="C163" t="s">
-        <v>9</v>
-      </c>
-      <c r="D163" t="s">
-        <v>19</v>
-      </c>
-      <c r="E163">
-        <v>12830</v>
-      </c>
-      <c r="F163">
-        <v>19</v>
-      </c>
-      <c r="H163" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="164" spans="1:8">
-      <c r="A164" t="s">
-        <v>8</v>
-      </c>
-      <c r="C164" t="s">
-        <v>9</v>
-      </c>
-      <c r="D164" t="s">
-        <v>21</v>
-      </c>
-      <c r="E164">
-        <v>25604</v>
-      </c>
-      <c r="F164">
-        <v>19</v>
-      </c>
-      <c r="H164" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="165" spans="1:8">
-      <c r="A165" t="s">
-        <v>8</v>
-      </c>
-      <c r="C165" t="s">
-        <v>9</v>
-      </c>
-      <c r="D165" t="s">
-        <v>22</v>
-      </c>
-      <c r="E165">
-        <v>3211</v>
-      </c>
-      <c r="F165">
-        <v>19</v>
-      </c>
-      <c r="H165" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8">
-      <c r="A166" t="s">
-        <v>8</v>
-      </c>
-      <c r="C166" t="s">
-        <v>9</v>
-      </c>
-      <c r="D166" t="s">
-        <v>26</v>
-      </c>
-      <c r="E166">
-        <v>136</v>
-      </c>
-      <c r="F166">
-        <v>19</v>
-      </c>
-      <c r="H166" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="167" spans="1:8">
-      <c r="A167" t="s">
-        <v>8</v>
-      </c>
-      <c r="C167" t="s">
-        <v>9</v>
-      </c>
-      <c r="D167" t="s">
-        <v>24</v>
-      </c>
-      <c r="E167">
-        <v>5870</v>
-      </c>
-      <c r="F167">
-        <v>19</v>
-      </c>
-      <c r="H167" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="168" spans="1:8">
-      <c r="A168" t="s">
-        <v>8</v>
-      </c>
-      <c r="C168" t="s">
-        <v>9</v>
-      </c>
-      <c r="D168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E168">
-        <v>136</v>
-      </c>
-      <c r="F168">
-        <v>19</v>
-      </c>
-      <c r="H168" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="169" spans="1:8">
-      <c r="A169" t="s">
-        <v>8</v>
-      </c>
-      <c r="C169" t="s">
-        <v>9</v>
-      </c>
-      <c r="D169" t="s">
-        <v>25</v>
-      </c>
-      <c r="E169">
-        <v>5870</v>
-      </c>
-      <c r="F169">
-        <v>19</v>
-      </c>
-      <c r="H169" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="170" spans="1:8">
-      <c r="A170" t="s">
-        <v>8</v>
-      </c>
-      <c r="C170" t="s">
-        <v>9</v>
-      </c>
-      <c r="D170" t="s">
-        <v>10</v>
-      </c>
-      <c r="E170">
-        <v>10749</v>
-      </c>
-      <c r="F170">
-        <v>19</v>
-      </c>
-      <c r="H170" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="171" spans="1:8">
-      <c r="A171" t="s">
-        <v>8</v>
-      </c>
-      <c r="C171" t="s">
-        <v>9</v>
-      </c>
-      <c r="D171" t="s">
-        <v>11</v>
-      </c>
-      <c r="E171">
-        <v>343</v>
-      </c>
-      <c r="F171">
-        <v>19</v>
-      </c>
-      <c r="H171" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="172" spans="1:8">
-      <c r="A172" t="s">
-        <v>8</v>
-      </c>
-      <c r="C172" t="s">
-        <v>9</v>
-      </c>
-      <c r="D172" t="s">
-        <v>12</v>
-      </c>
-      <c r="E172">
-        <v>19387</v>
-      </c>
-      <c r="F172">
-        <v>19</v>
-      </c>
-      <c r="H172" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="173" spans="1:8">
-      <c r="A173" t="s">
-        <v>8</v>
-      </c>
-      <c r="C173" t="s">
-        <v>9</v>
-      </c>
-      <c r="D173" t="s">
-        <v>23</v>
-      </c>
-      <c r="E173">
-        <v>2333</v>
-      </c>
-      <c r="F173">
-        <v>19</v>
-      </c>
-      <c r="H173" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="174" spans="1:8">
-      <c r="A174" t="s">
-        <v>8</v>
-      </c>
-      <c r="C174" t="s">
-        <v>9</v>
-      </c>
-      <c r="D174" t="s">
-        <v>13</v>
-      </c>
-      <c r="E174">
-        <v>17036</v>
-      </c>
-      <c r="F174">
-        <v>19</v>
-      </c>
-      <c r="H174" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="175" spans="1:8">
-      <c r="A175" t="s">
-        <v>8</v>
-      </c>
-      <c r="C175" t="s">
-        <v>9</v>
-      </c>
-      <c r="D175" t="s">
-        <v>14</v>
-      </c>
-      <c r="E175">
-        <v>25869</v>
-      </c>
-      <c r="F175">
-        <v>19</v>
-      </c>
-      <c r="H175" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="176" spans="1:8">
-      <c r="A176" t="s">
-        <v>8</v>
-      </c>
-      <c r="C176" t="s">
-        <v>9</v>
-      </c>
-      <c r="D176" t="s">
-        <v>15</v>
-      </c>
-      <c r="E176">
-        <v>9336</v>
-      </c>
-      <c r="F176">
-        <v>19</v>
-      </c>
-      <c r="H176" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="177" spans="1:8">
-      <c r="A177" t="s">
-        <v>8</v>
-      </c>
-      <c r="C177" t="s">
-        <v>9</v>
-      </c>
-      <c r="D177" t="s">
-        <v>16</v>
-      </c>
-      <c r="E177">
-        <v>10852</v>
-      </c>
-      <c r="F177">
-        <v>19</v>
-      </c>
-      <c r="H177" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="178" spans="1:8">
-      <c r="A178" t="s">
-        <v>8</v>
-      </c>
-      <c r="C178" t="s">
-        <v>9</v>
-      </c>
-      <c r="D178" t="s">
-        <v>17</v>
-      </c>
-      <c r="E178">
-        <v>8586</v>
-      </c>
-      <c r="F178">
-        <v>19</v>
-      </c>
-      <c r="H178" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="179" spans="1:8">
-      <c r="A179" t="s">
-        <v>8</v>
-      </c>
-      <c r="C179" t="s">
-        <v>9</v>
-      </c>
-      <c r="D179" t="s">
-        <v>18</v>
-      </c>
-      <c r="E179">
-        <v>11602</v>
-      </c>
-      <c r="F179">
-        <v>19</v>
-      </c>
-      <c r="H179" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="180" spans="1:8">
-      <c r="A180" t="s">
-        <v>8</v>
-      </c>
-      <c r="C180" t="s">
-        <v>9</v>
-      </c>
-      <c r="D180" t="s">
-        <v>19</v>
-      </c>
-      <c r="E180">
-        <v>14703</v>
-      </c>
-      <c r="F180">
-        <v>19</v>
-      </c>
-      <c r="H180" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="181" spans="1:8">
-      <c r="A181" t="s">
-        <v>8</v>
-      </c>
-      <c r="C181" t="s">
-        <v>9</v>
-      </c>
-      <c r="D181" t="s">
-        <v>21</v>
-      </c>
-      <c r="E181">
-        <v>25869</v>
-      </c>
-      <c r="F181">
-        <v>19</v>
-      </c>
-      <c r="H181" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="182" spans="1:8">
-      <c r="A182" t="s">
-        <v>8</v>
-      </c>
-      <c r="C182" t="s">
-        <v>9</v>
-      </c>
-      <c r="D182" t="s">
-        <v>22</v>
-      </c>
-      <c r="E182">
-        <v>3442</v>
-      </c>
-      <c r="F182">
-        <v>19</v>
-      </c>
-      <c r="H182" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="183" spans="1:8">
-      <c r="A183" t="s">
-        <v>8</v>
-      </c>
-      <c r="C183" t="s">
-        <v>9</v>
-      </c>
-      <c r="D183" t="s">
-        <v>26</v>
-      </c>
-      <c r="E183">
-        <v>764</v>
-      </c>
-      <c r="F183">
-        <v>19</v>
-      </c>
-      <c r="H183" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="184" spans="1:8">
-      <c r="A184" t="s">
-        <v>8</v>
-      </c>
-      <c r="C184" t="s">
-        <v>9</v>
-      </c>
-      <c r="D184" t="s">
-        <v>24</v>
-      </c>
-      <c r="E184">
-        <v>3962</v>
-      </c>
-      <c r="F184">
-        <v>19</v>
-      </c>
-      <c r="H184" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="185" spans="1:8">
-      <c r="A185" t="s">
-        <v>8</v>
-      </c>
-      <c r="C185" t="s">
-        <v>9</v>
-      </c>
-      <c r="D185" t="s">
-        <v>27</v>
-      </c>
-      <c r="E185">
-        <v>764</v>
-      </c>
-      <c r="F185">
-        <v>19</v>
-      </c>
-      <c r="H185" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="186" spans="1:8">
-      <c r="A186" t="s">
-        <v>8</v>
-      </c>
-      <c r="C186" t="s">
-        <v>9</v>
-      </c>
-      <c r="D186" t="s">
-        <v>25</v>
-      </c>
-      <c r="E186">
-        <v>3962</v>
-      </c>
-      <c r="F186">
-        <v>19</v>
-      </c>
-      <c r="H186" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code ready for teesting of QME, and its fluxos, direto, milk run e line haul
</commit_message>
<xml_diff>
--- a/Viajante/Template.xlsx
+++ b/Viajante/Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="35">
   <si>
     <t>COD FORNECEDOR</t>
   </si>
@@ -40,67 +40,49 @@
     <t>Mês</t>
   </si>
   <si>
-    <t>800002588</t>
+    <t>800006503</t>
   </si>
   <si>
-    <t>11568</t>
+    <t>70690</t>
   </si>
   <si>
     <t>1080</t>
   </si>
   <si>
-    <t>463488160</t>
+    <t>1002167600</t>
   </si>
   <si>
-    <t>463554420</t>
+    <t>1002167640</t>
   </si>
   <si>
-    <t>463587560</t>
+    <t>518359540</t>
   </si>
   <si>
-    <t>520420570</t>
+    <t>518442450</t>
   </si>
   <si>
-    <t>520420580</t>
+    <t>519499900</t>
   </si>
   <si>
-    <t>520445670</t>
+    <t>520404360</t>
   </si>
   <si>
-    <t>520542260</t>
+    <t>521286840</t>
   </si>
   <si>
-    <t>521095800</t>
+    <t>521286850</t>
   </si>
   <si>
-    <t>521582000</t>
+    <t>521286870</t>
   </si>
   <si>
-    <t>522310060</t>
+    <t>521286880</t>
   </si>
   <si>
-    <t>522315940</t>
+    <t>521427120</t>
   </si>
   <si>
-    <t>522315950</t>
-  </si>
-  <si>
-    <t>522370320</t>
-  </si>
-  <si>
-    <t>520337470</t>
-  </si>
-  <si>
-    <t>9872247780</t>
-  </si>
-  <si>
-    <t>9874623580</t>
-  </si>
-  <si>
-    <t>9872205180</t>
-  </si>
-  <si>
-    <t>9872255180</t>
+    <t>521491000</t>
   </si>
   <si>
     <t>Apr</t>
@@ -494,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -537,13 +519,13 @@
         <v>11</v>
       </c>
       <c r="E2">
-        <v>16016</v>
+        <v>2554</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -560,13 +542,13 @@
         <v>12</v>
       </c>
       <c r="E3">
-        <v>331</v>
+        <v>2554</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -583,13 +565,13 @@
         <v>13</v>
       </c>
       <c r="E4">
-        <v>18228</v>
+        <v>5107</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -606,13 +588,13 @@
         <v>14</v>
       </c>
       <c r="E5">
-        <v>10514</v>
+        <v>2554</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -629,13 +611,13 @@
         <v>15</v>
       </c>
       <c r="E6">
-        <v>23067</v>
+        <v>2554</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -652,13 +634,13 @@
         <v>16</v>
       </c>
       <c r="E7">
-        <v>11383</v>
+        <v>2554</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H7" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -675,13 +657,13 @@
         <v>17</v>
       </c>
       <c r="E8">
-        <v>7779</v>
+        <v>6514</v>
       </c>
       <c r="F8">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -698,13 +680,13 @@
         <v>18</v>
       </c>
       <c r="E9">
-        <v>11088</v>
+        <v>8460</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -721,13 +703,13 @@
         <v>19</v>
       </c>
       <c r="E10">
-        <v>8074</v>
+        <v>6514</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -744,13 +726,13 @@
         <v>20</v>
       </c>
       <c r="E11">
-        <v>10514</v>
+        <v>8460</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H11" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -767,13 +749,13 @@
         <v>21</v>
       </c>
       <c r="E12">
-        <v>411</v>
+        <v>14974</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -787,16 +769,16 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E13">
-        <v>23067</v>
+        <v>4049</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H13" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -810,16 +792,16 @@
         <v>10</v>
       </c>
       <c r="D14" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E14">
-        <v>3183</v>
+        <v>4049</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H14" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -833,16 +815,16 @@
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E15">
-        <v>22424</v>
+        <v>8098</v>
       </c>
       <c r="F15">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -856,16 +838,16 @@
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E16">
-        <v>330</v>
+        <v>4049</v>
       </c>
       <c r="F16">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H16" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -879,16 +861,16 @@
         <v>10</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E17">
-        <v>28470</v>
+        <v>4049</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H17" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -902,16 +884,16 @@
         <v>10</v>
       </c>
       <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18">
+        <v>4049</v>
+      </c>
+      <c r="F18">
+        <v>19</v>
+      </c>
+      <c r="H18" t="s">
         <v>24</v>
-      </c>
-      <c r="E18">
-        <v>550</v>
-      </c>
-      <c r="F18">
-        <v>4</v>
-      </c>
-      <c r="H18" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -925,16 +907,16 @@
         <v>10</v>
       </c>
       <c r="D19" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E19">
-        <v>17317</v>
+        <v>9738</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -948,16 +930,16 @@
         <v>10</v>
       </c>
       <c r="D20" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E20">
-        <v>36973</v>
+        <v>14737</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -971,16 +953,16 @@
         <v>10</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E21">
-        <v>16847</v>
+        <v>9738</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -994,16 +976,16 @@
         <v>10</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E22">
-        <v>12672</v>
+        <v>14737</v>
       </c>
       <c r="F22">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H22" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1017,16 +999,16 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E23">
-        <v>15049</v>
+        <v>24475</v>
       </c>
       <c r="F23">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H23" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1040,16 +1022,16 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E24">
-        <v>14470</v>
+        <v>2639</v>
       </c>
       <c r="F24">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H24" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1063,16 +1045,16 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E25">
-        <v>16767</v>
+        <v>2639</v>
       </c>
       <c r="F25">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1086,16 +1068,16 @@
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E26">
-        <v>138</v>
+        <v>5278</v>
       </c>
       <c r="F26">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H26" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1109,16 +1091,16 @@
         <v>10</v>
       </c>
       <c r="D27" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E27">
-        <v>36973</v>
+        <v>2639</v>
       </c>
       <c r="F27">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H27" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1132,16 +1114,16 @@
         <v>10</v>
       </c>
       <c r="D28" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E28">
-        <v>3600</v>
+        <v>2639</v>
       </c>
       <c r="F28">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H28" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1155,16 +1137,16 @@
         <v>10</v>
       </c>
       <c r="D29" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29">
+        <v>2639</v>
+      </c>
+      <c r="F29">
+        <v>19</v>
+      </c>
+      <c r="H29" t="s">
         <v>25</v>
-      </c>
-      <c r="E29">
-        <v>1476</v>
-      </c>
-      <c r="F29">
-        <v>4</v>
-      </c>
-      <c r="H29" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1178,16 +1160,16 @@
         <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E30">
-        <v>1476</v>
+        <v>8250</v>
       </c>
       <c r="F30">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H30" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1201,16 +1183,16 @@
         <v>10</v>
       </c>
       <c r="D31" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E31">
-        <v>15068</v>
+        <v>7444</v>
       </c>
       <c r="F31">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H31" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1224,16 +1206,16 @@
         <v>10</v>
       </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E32">
-        <v>95</v>
+        <v>8250</v>
       </c>
       <c r="F32">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H32" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1247,16 +1229,16 @@
         <v>10</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E33">
-        <v>18919</v>
+        <v>7444</v>
       </c>
       <c r="F33">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H33" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1270,16 +1252,16 @@
         <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E34">
-        <v>6043</v>
+        <v>15694</v>
       </c>
       <c r="F34">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H34" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1293,16 +1275,16 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E35">
-        <v>14008</v>
+        <v>2074</v>
       </c>
       <c r="F35">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H35" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1316,16 +1298,16 @@
         <v>10</v>
       </c>
       <c r="D36" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E36">
-        <v>23005</v>
+        <v>2074</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H36" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1339,16 +1321,16 @@
         <v>10</v>
       </c>
       <c r="D37" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E37">
-        <v>3691</v>
+        <v>4148</v>
       </c>
       <c r="F37">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H37" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1362,16 +1344,16 @@
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E38">
-        <v>8829</v>
+        <v>2074</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H38" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1385,16 +1367,16 @@
         <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>2864</v>
+        <v>2074</v>
       </c>
       <c r="F39">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H39" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -1408,16 +1390,16 @@
         <v>10</v>
       </c>
       <c r="D40" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>9656</v>
+        <v>2074</v>
       </c>
       <c r="F40">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H40" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -1431,16 +1413,16 @@
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E41">
-        <v>7965</v>
+        <v>5186</v>
       </c>
       <c r="F41">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H41" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -1454,16 +1436,16 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E42">
-        <v>23005</v>
+        <v>7155</v>
       </c>
       <c r="F42">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H42" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -1477,16 +1459,16 @@
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E43">
-        <v>107</v>
+        <v>5186</v>
       </c>
       <c r="F43">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H43" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -1500,16 +1482,16 @@
         <v>10</v>
       </c>
       <c r="D44" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E44">
-        <v>300</v>
+        <v>7155</v>
       </c>
       <c r="F44">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H44" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -1523,16 +1505,16 @@
         <v>10</v>
       </c>
       <c r="D45" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E45">
-        <v>7358</v>
+        <v>12341</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H45" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -1546,16 +1528,16 @@
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E46">
-        <v>300</v>
+        <v>623</v>
       </c>
       <c r="F46">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H46" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -1569,16 +1551,16 @@
         <v>10</v>
       </c>
       <c r="D47" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E47">
-        <v>7358</v>
+        <v>3157</v>
       </c>
       <c r="F47">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H47" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -1592,16 +1574,16 @@
         <v>10</v>
       </c>
       <c r="D48" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E48">
-        <v>14082</v>
+        <v>3157</v>
       </c>
       <c r="F48">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H48" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -1615,16 +1597,16 @@
         <v>10</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49">
-        <v>316</v>
+        <v>6314</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H49" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -1638,16 +1620,16 @@
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E50">
-        <v>15639</v>
+        <v>3157</v>
       </c>
       <c r="F50">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H50" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -1661,16 +1643,16 @@
         <v>10</v>
       </c>
       <c r="D51" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E51">
-        <v>9136</v>
+        <v>3157</v>
       </c>
       <c r="F51">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H51" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -1684,16 +1666,16 @@
         <v>10</v>
       </c>
       <c r="D52" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19144</v>
+        <v>3157</v>
       </c>
       <c r="F52">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H52" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -1707,16 +1689,16 @@
         <v>10</v>
       </c>
       <c r="D53" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E53">
-        <v>9832</v>
+        <v>7888</v>
       </c>
       <c r="F53">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H53" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -1730,16 +1712,16 @@
         <v>10</v>
       </c>
       <c r="D54" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E54">
-        <v>6477</v>
+        <v>10540</v>
       </c>
       <c r="F54">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H54" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -1753,16 +1735,16 @@
         <v>10</v>
       </c>
       <c r="D55" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E55">
-        <v>8950</v>
+        <v>7888</v>
       </c>
       <c r="F55">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H55" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -1776,16 +1758,16 @@
         <v>10</v>
       </c>
       <c r="D56" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E56">
-        <v>7359</v>
+        <v>10540</v>
       </c>
       <c r="F56">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H56" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -1799,16 +1781,16 @@
         <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E57">
-        <v>9136</v>
+        <v>18428</v>
       </c>
       <c r="F57">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H57" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -1822,16 +1804,16 @@
         <v>10</v>
       </c>
       <c r="D58" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E58">
-        <v>11</v>
+        <v>2960</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H58" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -1845,16 +1827,16 @@
         <v>10</v>
       </c>
       <c r="D59" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E59">
-        <v>19144</v>
+        <v>2960</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H59" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -1868,16 +1850,16 @@
         <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E60">
-        <v>1754</v>
+        <v>5920</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H60" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -1891,16 +1873,16 @@
         <v>10</v>
       </c>
       <c r="D61" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E61">
-        <v>42</v>
+        <v>2960</v>
       </c>
       <c r="F61">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H61" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -1914,16 +1896,16 @@
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="E62">
-        <v>42</v>
+        <v>2960</v>
       </c>
       <c r="F62">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H62" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -1937,16 +1919,16 @@
         <v>10</v>
       </c>
       <c r="D63" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E63">
-        <v>16606</v>
+        <v>2960</v>
       </c>
       <c r="F63">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H63" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -1960,16 +1942,16 @@
         <v>10</v>
       </c>
       <c r="D64" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E64">
-        <v>295</v>
+        <v>6186</v>
       </c>
       <c r="F64">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H64" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -1983,16 +1965,16 @@
         <v>10</v>
       </c>
       <c r="D65" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E65">
-        <v>24461</v>
+        <v>10704</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H65" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -2006,16 +1988,16 @@
         <v>10</v>
       </c>
       <c r="D66" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E66">
-        <v>7129</v>
+        <v>6186</v>
       </c>
       <c r="F66">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H66" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -2029,16 +2011,16 @@
         <v>10</v>
       </c>
       <c r="D67" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E67">
-        <v>17007</v>
+        <v>10704</v>
       </c>
       <c r="F67">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H67" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -2052,16 +2034,16 @@
         <v>10</v>
       </c>
       <c r="D68" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E68">
-        <v>21391</v>
+        <v>16890</v>
       </c>
       <c r="F68">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H68" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -2075,16 +2057,16 @@
         <v>10</v>
       </c>
       <c r="D69" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E69">
-        <v>4604</v>
+        <v>2705</v>
       </c>
       <c r="F69">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H69" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -2098,16 +2080,16 @@
         <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E70">
-        <v>7355</v>
+        <v>2705</v>
       </c>
       <c r="F70">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H70" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2121,16 +2103,16 @@
         <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E71">
-        <v>11959</v>
+        <v>5410</v>
       </c>
       <c r="F71">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H71" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -2144,16 +2126,16 @@
         <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E72">
-        <v>9878</v>
+        <v>2705</v>
       </c>
       <c r="F72">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H72" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -2167,16 +2149,16 @@
         <v>10</v>
       </c>
       <c r="D73" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E73">
-        <v>21391</v>
+        <v>2705</v>
       </c>
       <c r="F73">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H73" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -2190,16 +2172,16 @@
         <v>10</v>
       </c>
       <c r="D74" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E74">
-        <v>3016</v>
+        <v>2705</v>
       </c>
       <c r="F74">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H74" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -2213,16 +2195,16 @@
         <v>10</v>
       </c>
       <c r="D75" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E75">
-        <v>300</v>
+        <v>7728</v>
       </c>
       <c r="F75">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H75" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -2236,16 +2218,16 @@
         <v>10</v>
       </c>
       <c r="D76" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E76">
-        <v>8685</v>
+        <v>7823</v>
       </c>
       <c r="F76">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H76" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -2259,16 +2241,16 @@
         <v>10</v>
       </c>
       <c r="D77" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E77">
-        <v>300</v>
+        <v>7728</v>
       </c>
       <c r="F77">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H77" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -2282,16 +2264,16 @@
         <v>10</v>
       </c>
       <c r="D78" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E78">
-        <v>8685</v>
+        <v>7823</v>
       </c>
       <c r="F78">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H78" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -2305,16 +2287,16 @@
         <v>10</v>
       </c>
       <c r="D79" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E79">
-        <v>18433</v>
+        <v>15551</v>
       </c>
       <c r="F79">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H79" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -2328,16 +2310,16 @@
         <v>10</v>
       </c>
       <c r="D80" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E80">
-        <v>327</v>
+        <v>3735</v>
       </c>
       <c r="F80">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H80" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -2351,16 +2333,16 @@
         <v>10</v>
       </c>
       <c r="D81" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E81">
-        <v>23016</v>
+        <v>3735</v>
       </c>
       <c r="F81">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H81" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -2374,16 +2356,16 @@
         <v>10</v>
       </c>
       <c r="D82" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E82">
-        <v>151</v>
+        <v>7470</v>
       </c>
       <c r="F82">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H82" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -2400,13 +2382,13 @@
         <v>14</v>
       </c>
       <c r="E83">
-        <v>10864</v>
+        <v>3735</v>
       </c>
       <c r="F83">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H83" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -2423,13 +2405,13 @@
         <v>15</v>
       </c>
       <c r="E84">
-        <v>24385</v>
+        <v>3735</v>
       </c>
       <c r="F84">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H84" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -2446,13 +2428,13 @@
         <v>16</v>
       </c>
       <c r="E85">
-        <v>13190</v>
+        <v>3735</v>
       </c>
       <c r="F85">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H85" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -2469,13 +2451,13 @@
         <v>17</v>
       </c>
       <c r="E86">
-        <v>8218</v>
+        <v>9405</v>
       </c>
       <c r="F86">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H86" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -2492,13 +2474,13 @@
         <v>18</v>
       </c>
       <c r="E87">
-        <v>11218</v>
+        <v>11879</v>
       </c>
       <c r="F87">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H87" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -2515,13 +2497,13 @@
         <v>19</v>
       </c>
       <c r="E88">
-        <v>10190</v>
+        <v>9405</v>
       </c>
       <c r="F88">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H88" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -2538,13 +2520,13 @@
         <v>20</v>
       </c>
       <c r="E89">
-        <v>10713</v>
+        <v>11879</v>
       </c>
       <c r="F89">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H89" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -2561,13 +2543,13 @@
         <v>21</v>
       </c>
       <c r="E90">
-        <v>125</v>
+        <v>21284</v>
       </c>
       <c r="F90">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H90" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -2581,16 +2563,16 @@
         <v>10</v>
       </c>
       <c r="D91" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E91">
-        <v>24385</v>
+        <v>3888</v>
       </c>
       <c r="F91">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H91" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -2604,16 +2586,16 @@
         <v>10</v>
       </c>
       <c r="D92" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E92">
-        <v>3717</v>
+        <v>3888</v>
       </c>
       <c r="F92">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H92" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -2627,16 +2609,16 @@
         <v>10</v>
       </c>
       <c r="D93" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E93">
-        <v>276</v>
+        <v>7777</v>
       </c>
       <c r="F93">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H93" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -2650,16 +2632,16 @@
         <v>10</v>
       </c>
       <c r="D94" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E94">
-        <v>276</v>
+        <v>3888</v>
       </c>
       <c r="F94">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H94" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -2673,16 +2655,16 @@
         <v>10</v>
       </c>
       <c r="D95" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E95">
-        <v>16778</v>
+        <v>3888</v>
       </c>
       <c r="F95">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H95" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -2696,16 +2678,16 @@
         <v>10</v>
       </c>
       <c r="D96" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E96">
-        <v>96</v>
+        <v>3888</v>
       </c>
       <c r="F96">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H96" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -2719,16 +2701,16 @@
         <v>10</v>
       </c>
       <c r="D97" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E97">
-        <v>19772</v>
+        <v>9161</v>
       </c>
       <c r="F97">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H97" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -2742,16 +2724,16 @@
         <v>10</v>
       </c>
       <c r="D98" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E98">
-        <v>7</v>
+        <v>12565</v>
       </c>
       <c r="F98">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H98" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -2765,16 +2747,16 @@
         <v>10</v>
       </c>
       <c r="D99" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E99">
-        <v>11575</v>
+        <v>9161</v>
       </c>
       <c r="F99">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H99" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="100" spans="1:8">
@@ -2788,16 +2770,16 @@
         <v>10</v>
       </c>
       <c r="D100" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E100">
-        <v>25545</v>
+        <v>12565</v>
       </c>
       <c r="F100">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H100" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -2811,16 +2793,16 @@
         <v>10</v>
       </c>
       <c r="D101" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E101">
-        <v>12013</v>
+        <v>21726</v>
       </c>
       <c r="F101">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H101" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -2834,16 +2816,16 @@
         <v>10</v>
       </c>
       <c r="D102" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E102">
-        <v>9285</v>
+        <v>3784</v>
       </c>
       <c r="F102">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H102" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -2857,16 +2839,16 @@
         <v>10</v>
       </c>
       <c r="D103" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E103">
-        <v>12111</v>
+        <v>3784</v>
       </c>
       <c r="F103">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H103" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -2880,16 +2862,16 @@
         <v>10</v>
       </c>
       <c r="D104" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E104">
-        <v>9187</v>
+        <v>7568</v>
       </c>
       <c r="F104">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H104" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -2903,16 +2885,16 @@
         <v>10</v>
       </c>
       <c r="D105" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E105">
-        <v>11568</v>
+        <v>3784</v>
       </c>
       <c r="F105">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H105" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -2926,16 +2908,16 @@
         <v>10</v>
       </c>
       <c r="D106" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E106">
-        <v>121</v>
+        <v>3784</v>
       </c>
       <c r="F106">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H106" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -2949,16 +2931,16 @@
         <v>10</v>
       </c>
       <c r="D107" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E107">
-        <v>25545</v>
+        <v>3784</v>
       </c>
       <c r="F107">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H107" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -2972,16 +2954,16 @@
         <v>10</v>
       </c>
       <c r="D108" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E108">
-        <v>1831</v>
+        <v>7869</v>
       </c>
       <c r="F108">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H108" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -2995,16 +2977,16 @@
         <v>10</v>
       </c>
       <c r="D109" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E109">
-        <v>30</v>
+        <v>14381</v>
       </c>
       <c r="F109">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H109" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -3018,16 +3000,16 @@
         <v>10</v>
       </c>
       <c r="D110" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E110">
-        <v>30</v>
+        <v>7869</v>
       </c>
       <c r="F110">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H110" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -3041,16 +3023,16 @@
         <v>10</v>
       </c>
       <c r="D111" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E111">
-        <v>20272</v>
+        <v>14381</v>
       </c>
       <c r="F111">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H111" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -3064,16 +3046,16 @@
         <v>10</v>
       </c>
       <c r="D112" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E112">
-        <v>267</v>
+        <v>22250</v>
       </c>
       <c r="F112">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H112" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -3087,16 +3069,16 @@
         <v>10</v>
       </c>
       <c r="D113" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E113">
-        <v>24924</v>
+        <v>3302</v>
       </c>
       <c r="F113">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H113" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -3110,16 +3092,16 @@
         <v>10</v>
       </c>
       <c r="D114" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E114">
-        <v>15572</v>
+        <v>3302</v>
       </c>
       <c r="F114">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H114" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -3133,16 +3115,16 @@
         <v>10</v>
       </c>
       <c r="D115" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E115">
-        <v>32977</v>
+        <v>6604</v>
       </c>
       <c r="F115">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H115" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="116" spans="1:8">
@@ -3156,16 +3138,16 @@
         <v>10</v>
       </c>
       <c r="D116" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E116">
-        <v>16099</v>
+        <v>3302</v>
       </c>
       <c r="F116">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H116" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="117" spans="1:8">
@@ -3179,16 +3161,16 @@
         <v>10</v>
       </c>
       <c r="D117" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E117">
-        <v>10916</v>
+        <v>3302</v>
       </c>
       <c r="F117">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H117" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="118" spans="1:8">
@@ -3202,16 +3184,16 @@
         <v>10</v>
       </c>
       <c r="D118" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E118">
-        <v>15010</v>
+        <v>3302</v>
       </c>
       <c r="F118">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H118" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="119" spans="1:8">
@@ -3225,16 +3207,16 @@
         <v>10</v>
       </c>
       <c r="D119" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E119">
-        <v>12005</v>
+        <v>7873</v>
       </c>
       <c r="F119">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H119" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="120" spans="1:8">
@@ -3248,16 +3230,16 @@
         <v>10</v>
       </c>
       <c r="D120" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E120">
-        <v>15572</v>
+        <v>10991</v>
       </c>
       <c r="F120">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H120" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="121" spans="1:8">
@@ -3271,16 +3253,16 @@
         <v>10</v>
       </c>
       <c r="D121" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E121">
-        <v>32977</v>
+        <v>7873</v>
       </c>
       <c r="F121">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H121" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="122" spans="1:8">
@@ -3294,16 +3276,16 @@
         <v>10</v>
       </c>
       <c r="D122" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E122">
-        <v>3132</v>
+        <v>10991</v>
       </c>
       <c r="F122">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H122" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="123" spans="1:8">
@@ -3317,16 +3299,16 @@
         <v>10</v>
       </c>
       <c r="D123" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E123">
-        <v>23264</v>
+        <v>18864</v>
       </c>
       <c r="F123">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H123" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="124" spans="1:8">
@@ -3340,16 +3322,16 @@
         <v>10</v>
       </c>
       <c r="D124" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E124">
-        <v>492</v>
+        <v>3212</v>
       </c>
       <c r="F124">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H124" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:8">
@@ -3363,16 +3345,16 @@
         <v>10</v>
       </c>
       <c r="D125" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E125">
-        <v>29845</v>
+        <v>3212</v>
       </c>
       <c r="F125">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H125" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="126" spans="1:8">
@@ -3386,16 +3368,16 @@
         <v>10</v>
       </c>
       <c r="D126" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E126">
-        <v>17622</v>
+        <v>6424</v>
       </c>
       <c r="F126">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H126" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:8">
@@ -3409,16 +3391,16 @@
         <v>10</v>
       </c>
       <c r="D127" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E127">
-        <v>31611</v>
+        <v>3212</v>
       </c>
       <c r="F127">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H127" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="128" spans="1:8">
@@ -3432,16 +3414,16 @@
         <v>10</v>
       </c>
       <c r="D128" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E128">
-        <v>16937</v>
+        <v>3212</v>
       </c>
       <c r="F128">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H128" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="129" spans="1:8">
@@ -3455,16 +3437,16 @@
         <v>10</v>
       </c>
       <c r="D129" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E129">
-        <v>11586</v>
+        <v>3212</v>
       </c>
       <c r="F129">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H129" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="130" spans="1:8">
@@ -3478,16 +3460,16 @@
         <v>10</v>
       </c>
       <c r="D130" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E130">
-        <v>15209</v>
+        <v>10490</v>
       </c>
       <c r="F130">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H130" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="131" spans="1:8">
@@ -3501,16 +3483,16 @@
         <v>10</v>
       </c>
       <c r="D131" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E131">
-        <v>13314</v>
+        <v>7637</v>
       </c>
       <c r="F131">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H131" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="132" spans="1:8">
@@ -3524,16 +3506,16 @@
         <v>10</v>
       </c>
       <c r="D132" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E132">
-        <v>17622</v>
+        <v>10490</v>
       </c>
       <c r="F132">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H132" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -3547,16 +3529,16 @@
         <v>10</v>
       </c>
       <c r="D133" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E133">
-        <v>525</v>
+        <v>7637</v>
       </c>
       <c r="F133">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H133" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="134" spans="1:8">
@@ -3570,1212 +3552,16 @@
         <v>10</v>
       </c>
       <c r="D134" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E134">
-        <v>31611</v>
+        <v>18127</v>
       </c>
       <c r="F134">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H134" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="135" spans="1:8">
-      <c r="A135" t="s">
-        <v>8</v>
-      </c>
-      <c r="B135" t="s">
-        <v>9</v>
-      </c>
-      <c r="C135" t="s">
-        <v>10</v>
-      </c>
-      <c r="D135" t="s">
-        <v>23</v>
-      </c>
-      <c r="E135">
-        <v>4688</v>
-      </c>
-      <c r="F135">
-        <v>4</v>
-      </c>
-      <c r="H135" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="136" spans="1:8">
-      <c r="A136" t="s">
-        <v>8</v>
-      </c>
-      <c r="B136" t="s">
-        <v>9</v>
-      </c>
-      <c r="C136" t="s">
-        <v>10</v>
-      </c>
-      <c r="D136" t="s">
-        <v>11</v>
-      </c>
-      <c r="E136">
-        <v>21786</v>
-      </c>
-      <c r="F136">
-        <v>4</v>
-      </c>
-      <c r="H136" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8">
-      <c r="A137" t="s">
-        <v>8</v>
-      </c>
-      <c r="B137" t="s">
-        <v>9</v>
-      </c>
-      <c r="C137" t="s">
-        <v>10</v>
-      </c>
-      <c r="D137" t="s">
-        <v>12</v>
-      </c>
-      <c r="E137">
-        <v>555</v>
-      </c>
-      <c r="F137">
-        <v>4</v>
-      </c>
-      <c r="H137" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8">
-      <c r="A138" t="s">
-        <v>8</v>
-      </c>
-      <c r="B138" t="s">
-        <v>9</v>
-      </c>
-      <c r="C138" t="s">
-        <v>10</v>
-      </c>
-      <c r="D138" t="s">
-        <v>13</v>
-      </c>
-      <c r="E138">
-        <v>33114</v>
-      </c>
-      <c r="F138">
-        <v>4</v>
-      </c>
-      <c r="H138" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="139" spans="1:8">
-      <c r="A139" t="s">
-        <v>8</v>
-      </c>
-      <c r="B139" t="s">
-        <v>9</v>
-      </c>
-      <c r="C139" t="s">
-        <v>10</v>
-      </c>
-      <c r="D139" t="s">
-        <v>24</v>
-      </c>
-      <c r="E139">
-        <v>8449</v>
-      </c>
-      <c r="F139">
-        <v>4</v>
-      </c>
-      <c r="H139" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="140" spans="1:8">
-      <c r="A140" t="s">
-        <v>8</v>
-      </c>
-      <c r="B140" t="s">
-        <v>9</v>
-      </c>
-      <c r="C140" t="s">
-        <v>10</v>
-      </c>
-      <c r="D140" t="s">
-        <v>14</v>
-      </c>
-      <c r="E140">
-        <v>20744</v>
-      </c>
-      <c r="F140">
-        <v>4</v>
-      </c>
-      <c r="H140" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="141" spans="1:8">
-      <c r="A141" t="s">
-        <v>8</v>
-      </c>
-      <c r="B141" t="s">
-        <v>9</v>
-      </c>
-      <c r="C141" t="s">
-        <v>10</v>
-      </c>
-      <c r="D141" t="s">
-        <v>15</v>
-      </c>
-      <c r="E141">
-        <v>28147</v>
-      </c>
-      <c r="F141">
-        <v>4</v>
-      </c>
-      <c r="H141" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8">
-      <c r="A142" t="s">
-        <v>8</v>
-      </c>
-      <c r="B142" t="s">
-        <v>9</v>
-      </c>
-      <c r="C142" t="s">
-        <v>10</v>
-      </c>
-      <c r="D142" t="s">
-        <v>16</v>
-      </c>
-      <c r="E142">
-        <v>5205</v>
-      </c>
-      <c r="F142">
-        <v>4</v>
-      </c>
-      <c r="H142" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="143" spans="1:8">
-      <c r="A143" t="s">
-        <v>8</v>
-      </c>
-      <c r="B143" t="s">
-        <v>9</v>
-      </c>
-      <c r="C143" t="s">
-        <v>10</v>
-      </c>
-      <c r="D143" t="s">
-        <v>17</v>
-      </c>
-      <c r="E143">
-        <v>13432</v>
-      </c>
-      <c r="F143">
-        <v>4</v>
-      </c>
-      <c r="H143" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="144" spans="1:8">
-      <c r="A144" t="s">
-        <v>8</v>
-      </c>
-      <c r="B144" t="s">
-        <v>9</v>
-      </c>
-      <c r="C144" t="s">
-        <v>10</v>
-      </c>
-      <c r="D144" t="s">
-        <v>18</v>
-      </c>
-      <c r="E144">
-        <v>4751</v>
-      </c>
-      <c r="F144">
-        <v>4</v>
-      </c>
-      <c r="H144" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="145" spans="1:8">
-      <c r="A145" t="s">
-        <v>8</v>
-      </c>
-      <c r="B145" t="s">
-        <v>9</v>
-      </c>
-      <c r="C145" t="s">
-        <v>10</v>
-      </c>
-      <c r="D145" t="s">
-        <v>19</v>
-      </c>
-      <c r="E145">
-        <v>13886</v>
-      </c>
-      <c r="F145">
-        <v>4</v>
-      </c>
-      <c r="H145" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="146" spans="1:8">
-      <c r="A146" t="s">
-        <v>8</v>
-      </c>
-      <c r="B146" t="s">
-        <v>9</v>
-      </c>
-      <c r="C146" t="s">
-        <v>10</v>
-      </c>
-      <c r="D146" t="s">
-        <v>20</v>
-      </c>
-      <c r="E146">
-        <v>12295</v>
-      </c>
-      <c r="F146">
-        <v>4</v>
-      </c>
-      <c r="H146" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="147" spans="1:8">
-      <c r="A147" t="s">
-        <v>8</v>
-      </c>
-      <c r="B147" t="s">
-        <v>9</v>
-      </c>
-      <c r="C147" t="s">
-        <v>10</v>
-      </c>
-      <c r="D147" t="s">
-        <v>22</v>
-      </c>
-      <c r="E147">
-        <v>28147</v>
-      </c>
-      <c r="F147">
-        <v>4</v>
-      </c>
-      <c r="H147" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8">
-      <c r="A148" t="s">
-        <v>8</v>
-      </c>
-      <c r="B148" t="s">
-        <v>9</v>
-      </c>
-      <c r="C148" t="s">
-        <v>10</v>
-      </c>
-      <c r="D148" t="s">
-        <v>23</v>
-      </c>
-      <c r="E148">
-        <v>5821</v>
-      </c>
-      <c r="F148">
-        <v>4</v>
-      </c>
-      <c r="H148" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="149" spans="1:8">
-      <c r="A149" t="s">
-        <v>8</v>
-      </c>
-      <c r="B149" t="s">
-        <v>9</v>
-      </c>
-      <c r="C149" t="s">
-        <v>10</v>
-      </c>
-      <c r="D149" t="s">
-        <v>27</v>
-      </c>
-      <c r="E149">
-        <v>300</v>
-      </c>
-      <c r="F149">
-        <v>4</v>
-      </c>
-      <c r="H149" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="150" spans="1:8">
-      <c r="A150" t="s">
-        <v>8</v>
-      </c>
-      <c r="B150" t="s">
-        <v>9</v>
-      </c>
-      <c r="C150" t="s">
-        <v>10</v>
-      </c>
-      <c r="D150" t="s">
-        <v>25</v>
-      </c>
-      <c r="E150">
-        <v>10760</v>
-      </c>
-      <c r="F150">
-        <v>4</v>
-      </c>
-      <c r="H150" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8">
-      <c r="A151" t="s">
-        <v>8</v>
-      </c>
-      <c r="B151" t="s">
-        <v>9</v>
-      </c>
-      <c r="C151" t="s">
-        <v>10</v>
-      </c>
-      <c r="D151" t="s">
-        <v>28</v>
-      </c>
-      <c r="E151">
-        <v>300</v>
-      </c>
-      <c r="F151">
-        <v>4</v>
-      </c>
-      <c r="H151" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8">
-      <c r="A152" t="s">
-        <v>8</v>
-      </c>
-      <c r="B152" t="s">
-        <v>9</v>
-      </c>
-      <c r="C152" t="s">
-        <v>10</v>
-      </c>
-      <c r="D152" t="s">
-        <v>26</v>
-      </c>
-      <c r="E152">
-        <v>10760</v>
-      </c>
-      <c r="F152">
-        <v>4</v>
-      </c>
-      <c r="H152" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8">
-      <c r="A153" t="s">
-        <v>8</v>
-      </c>
-      <c r="B153" t="s">
-        <v>9</v>
-      </c>
-      <c r="C153" t="s">
-        <v>10</v>
-      </c>
-      <c r="D153" t="s">
-        <v>11</v>
-      </c>
-      <c r="E153">
-        <v>17433</v>
-      </c>
-      <c r="F153">
-        <v>4</v>
-      </c>
-      <c r="H153" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8">
-      <c r="A154" t="s">
-        <v>8</v>
-      </c>
-      <c r="B154" t="s">
-        <v>9</v>
-      </c>
-      <c r="C154" t="s">
-        <v>10</v>
-      </c>
-      <c r="D154" t="s">
-        <v>12</v>
-      </c>
-      <c r="E154">
-        <v>245</v>
-      </c>
-      <c r="F154">
-        <v>4</v>
-      </c>
-      <c r="H154" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="155" spans="1:8">
-      <c r="A155" t="s">
-        <v>8</v>
-      </c>
-      <c r="B155" t="s">
-        <v>9</v>
-      </c>
-      <c r="C155" t="s">
-        <v>10</v>
-      </c>
-      <c r="D155" t="s">
-        <v>13</v>
-      </c>
-      <c r="E155">
-        <v>25359</v>
-      </c>
-      <c r="F155">
-        <v>4</v>
-      </c>
-      <c r="H155" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8">
-      <c r="A156" t="s">
-        <v>8</v>
-      </c>
-      <c r="B156" t="s">
-        <v>9</v>
-      </c>
-      <c r="C156" t="s">
-        <v>10</v>
-      </c>
-      <c r="D156" t="s">
-        <v>24</v>
-      </c>
-      <c r="E156">
-        <v>4436</v>
-      </c>
-      <c r="F156">
-        <v>4</v>
-      </c>
-      <c r="H156" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8">
-      <c r="A157" t="s">
-        <v>8</v>
-      </c>
-      <c r="B157" t="s">
-        <v>9</v>
-      </c>
-      <c r="C157" t="s">
-        <v>10</v>
-      </c>
-      <c r="D157" t="s">
-        <v>14</v>
-      </c>
-      <c r="E157">
-        <v>17266</v>
-      </c>
-      <c r="F157">
-        <v>4</v>
-      </c>
-      <c r="H157" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="158" spans="1:8">
-      <c r="A158" t="s">
-        <v>8</v>
-      </c>
-      <c r="B158" t="s">
-        <v>9</v>
-      </c>
-      <c r="C158" t="s">
-        <v>10</v>
-      </c>
-      <c r="D158" t="s">
-        <v>15</v>
-      </c>
-      <c r="E158">
-        <v>25604</v>
-      </c>
-      <c r="F158">
-        <v>4</v>
-      </c>
-      <c r="H158" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="159" spans="1:8">
-      <c r="A159" t="s">
-        <v>8</v>
-      </c>
-      <c r="B159" t="s">
-        <v>9</v>
-      </c>
-      <c r="C159" t="s">
-        <v>10</v>
-      </c>
-      <c r="D159" t="s">
-        <v>16</v>
-      </c>
-      <c r="E159">
-        <v>6920</v>
-      </c>
-      <c r="F159">
-        <v>4</v>
-      </c>
-      <c r="H159" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="160" spans="1:8">
-      <c r="A160" t="s">
-        <v>8</v>
-      </c>
-      <c r="B160" t="s">
-        <v>9</v>
-      </c>
-      <c r="C160" t="s">
-        <v>10</v>
-      </c>
-      <c r="D160" t="s">
-        <v>17</v>
-      </c>
-      <c r="E160">
-        <v>10844</v>
-      </c>
-      <c r="F160">
-        <v>4</v>
-      </c>
-      <c r="H160" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="161" spans="1:8">
-      <c r="A161" t="s">
-        <v>8</v>
-      </c>
-      <c r="B161" t="s">
-        <v>9</v>
-      </c>
-      <c r="C161" t="s">
-        <v>10</v>
-      </c>
-      <c r="D161" t="s">
-        <v>18</v>
-      </c>
-      <c r="E161">
-        <v>5932</v>
-      </c>
-      <c r="F161">
-        <v>4</v>
-      </c>
-      <c r="H161" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="162" spans="1:8">
-      <c r="A162" t="s">
-        <v>8</v>
-      </c>
-      <c r="B162" t="s">
-        <v>9</v>
-      </c>
-      <c r="C162" t="s">
-        <v>10</v>
-      </c>
-      <c r="D162" t="s">
-        <v>19</v>
-      </c>
-      <c r="E162">
-        <v>11832</v>
-      </c>
-      <c r="F162">
-        <v>4</v>
-      </c>
-      <c r="H162" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="163" spans="1:8">
-      <c r="A163" t="s">
-        <v>8</v>
-      </c>
-      <c r="B163" t="s">
-        <v>9</v>
-      </c>
-      <c r="C163" t="s">
-        <v>10</v>
-      </c>
-      <c r="D163" t="s">
-        <v>20</v>
-      </c>
-      <c r="E163">
-        <v>12830</v>
-      </c>
-      <c r="F163">
-        <v>4</v>
-      </c>
-      <c r="H163" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="164" spans="1:8">
-      <c r="A164" t="s">
-        <v>8</v>
-      </c>
-      <c r="B164" t="s">
-        <v>9</v>
-      </c>
-      <c r="C164" t="s">
-        <v>10</v>
-      </c>
-      <c r="D164" t="s">
-        <v>22</v>
-      </c>
-      <c r="E164">
-        <v>25604</v>
-      </c>
-      <c r="F164">
-        <v>4</v>
-      </c>
-      <c r="H164" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="165" spans="1:8">
-      <c r="A165" t="s">
-        <v>8</v>
-      </c>
-      <c r="B165" t="s">
-        <v>9</v>
-      </c>
-      <c r="C165" t="s">
-        <v>10</v>
-      </c>
-      <c r="D165" t="s">
-        <v>23</v>
-      </c>
-      <c r="E165">
-        <v>3211</v>
-      </c>
-      <c r="F165">
-        <v>4</v>
-      </c>
-      <c r="H165" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8">
-      <c r="A166" t="s">
-        <v>8</v>
-      </c>
-      <c r="B166" t="s">
-        <v>9</v>
-      </c>
-      <c r="C166" t="s">
-        <v>10</v>
-      </c>
-      <c r="D166" t="s">
-        <v>27</v>
-      </c>
-      <c r="E166">
-        <v>136</v>
-      </c>
-      <c r="F166">
-        <v>4</v>
-      </c>
-      <c r="H166" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="167" spans="1:8">
-      <c r="A167" t="s">
-        <v>8</v>
-      </c>
-      <c r="B167" t="s">
-        <v>9</v>
-      </c>
-      <c r="C167" t="s">
-        <v>10</v>
-      </c>
-      <c r="D167" t="s">
-        <v>25</v>
-      </c>
-      <c r="E167">
-        <v>5870</v>
-      </c>
-      <c r="F167">
-        <v>4</v>
-      </c>
-      <c r="H167" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="168" spans="1:8">
-      <c r="A168" t="s">
-        <v>8</v>
-      </c>
-      <c r="B168" t="s">
-        <v>9</v>
-      </c>
-      <c r="C168" t="s">
-        <v>10</v>
-      </c>
-      <c r="D168" t="s">
-        <v>28</v>
-      </c>
-      <c r="E168">
-        <v>136</v>
-      </c>
-      <c r="F168">
-        <v>4</v>
-      </c>
-      <c r="H168" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="169" spans="1:8">
-      <c r="A169" t="s">
-        <v>8</v>
-      </c>
-      <c r="B169" t="s">
-        <v>9</v>
-      </c>
-      <c r="C169" t="s">
-        <v>10</v>
-      </c>
-      <c r="D169" t="s">
-        <v>26</v>
-      </c>
-      <c r="E169">
-        <v>5870</v>
-      </c>
-      <c r="F169">
-        <v>4</v>
-      </c>
-      <c r="H169" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="170" spans="1:8">
-      <c r="A170" t="s">
-        <v>8</v>
-      </c>
-      <c r="B170" t="s">
-        <v>9</v>
-      </c>
-      <c r="C170" t="s">
-        <v>10</v>
-      </c>
-      <c r="D170" t="s">
-        <v>11</v>
-      </c>
-      <c r="E170">
-        <v>10749</v>
-      </c>
-      <c r="F170">
-        <v>4</v>
-      </c>
-      <c r="H170" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="171" spans="1:8">
-      <c r="A171" t="s">
-        <v>8</v>
-      </c>
-      <c r="B171" t="s">
-        <v>9</v>
-      </c>
-      <c r="C171" t="s">
-        <v>10</v>
-      </c>
-      <c r="D171" t="s">
-        <v>12</v>
-      </c>
-      <c r="E171">
-        <v>343</v>
-      </c>
-      <c r="F171">
-        <v>4</v>
-      </c>
-      <c r="H171" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="172" spans="1:8">
-      <c r="A172" t="s">
-        <v>8</v>
-      </c>
-      <c r="B172" t="s">
-        <v>9</v>
-      </c>
-      <c r="C172" t="s">
-        <v>10</v>
-      </c>
-      <c r="D172" t="s">
-        <v>13</v>
-      </c>
-      <c r="E172">
-        <v>19387</v>
-      </c>
-      <c r="F172">
-        <v>4</v>
-      </c>
-      <c r="H172" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="173" spans="1:8">
-      <c r="A173" t="s">
-        <v>8</v>
-      </c>
-      <c r="B173" t="s">
-        <v>9</v>
-      </c>
-      <c r="C173" t="s">
-        <v>10</v>
-      </c>
-      <c r="D173" t="s">
-        <v>24</v>
-      </c>
-      <c r="E173">
-        <v>2333</v>
-      </c>
-      <c r="F173">
-        <v>4</v>
-      </c>
-      <c r="H173" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="174" spans="1:8">
-      <c r="A174" t="s">
-        <v>8</v>
-      </c>
-      <c r="B174" t="s">
-        <v>9</v>
-      </c>
-      <c r="C174" t="s">
-        <v>10</v>
-      </c>
-      <c r="D174" t="s">
-        <v>14</v>
-      </c>
-      <c r="E174">
-        <v>17036</v>
-      </c>
-      <c r="F174">
-        <v>4</v>
-      </c>
-      <c r="H174" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="175" spans="1:8">
-      <c r="A175" t="s">
-        <v>8</v>
-      </c>
-      <c r="B175" t="s">
-        <v>9</v>
-      </c>
-      <c r="C175" t="s">
-        <v>10</v>
-      </c>
-      <c r="D175" t="s">
-        <v>15</v>
-      </c>
-      <c r="E175">
-        <v>25869</v>
-      </c>
-      <c r="F175">
-        <v>4</v>
-      </c>
-      <c r="H175" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="176" spans="1:8">
-      <c r="A176" t="s">
-        <v>8</v>
-      </c>
-      <c r="B176" t="s">
-        <v>9</v>
-      </c>
-      <c r="C176" t="s">
-        <v>10</v>
-      </c>
-      <c r="D176" t="s">
-        <v>16</v>
-      </c>
-      <c r="E176">
-        <v>9336</v>
-      </c>
-      <c r="F176">
-        <v>4</v>
-      </c>
-      <c r="H176" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="177" spans="1:8">
-      <c r="A177" t="s">
-        <v>8</v>
-      </c>
-      <c r="B177" t="s">
-        <v>9</v>
-      </c>
-      <c r="C177" t="s">
-        <v>10</v>
-      </c>
-      <c r="D177" t="s">
-        <v>17</v>
-      </c>
-      <c r="E177">
-        <v>10852</v>
-      </c>
-      <c r="F177">
-        <v>4</v>
-      </c>
-      <c r="H177" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="178" spans="1:8">
-      <c r="A178" t="s">
-        <v>8</v>
-      </c>
-      <c r="B178" t="s">
-        <v>9</v>
-      </c>
-      <c r="C178" t="s">
-        <v>10</v>
-      </c>
-      <c r="D178" t="s">
-        <v>18</v>
-      </c>
-      <c r="E178">
-        <v>8586</v>
-      </c>
-      <c r="F178">
-        <v>4</v>
-      </c>
-      <c r="H178" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="179" spans="1:8">
-      <c r="A179" t="s">
-        <v>8</v>
-      </c>
-      <c r="B179" t="s">
-        <v>9</v>
-      </c>
-      <c r="C179" t="s">
-        <v>10</v>
-      </c>
-      <c r="D179" t="s">
-        <v>19</v>
-      </c>
-      <c r="E179">
-        <v>11602</v>
-      </c>
-      <c r="F179">
-        <v>4</v>
-      </c>
-      <c r="H179" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="180" spans="1:8">
-      <c r="A180" t="s">
-        <v>8</v>
-      </c>
-      <c r="B180" t="s">
-        <v>9</v>
-      </c>
-      <c r="C180" t="s">
-        <v>10</v>
-      </c>
-      <c r="D180" t="s">
-        <v>20</v>
-      </c>
-      <c r="E180">
-        <v>14703</v>
-      </c>
-      <c r="F180">
-        <v>4</v>
-      </c>
-      <c r="H180" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="181" spans="1:8">
-      <c r="A181" t="s">
-        <v>8</v>
-      </c>
-      <c r="B181" t="s">
-        <v>9</v>
-      </c>
-      <c r="C181" t="s">
-        <v>10</v>
-      </c>
-      <c r="D181" t="s">
-        <v>22</v>
-      </c>
-      <c r="E181">
-        <v>25869</v>
-      </c>
-      <c r="F181">
-        <v>4</v>
-      </c>
-      <c r="H181" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="182" spans="1:8">
-      <c r="A182" t="s">
-        <v>8</v>
-      </c>
-      <c r="B182" t="s">
-        <v>9</v>
-      </c>
-      <c r="C182" t="s">
-        <v>10</v>
-      </c>
-      <c r="D182" t="s">
-        <v>23</v>
-      </c>
-      <c r="E182">
-        <v>3442</v>
-      </c>
-      <c r="F182">
-        <v>4</v>
-      </c>
-      <c r="H182" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="183" spans="1:8">
-      <c r="A183" t="s">
-        <v>8</v>
-      </c>
-      <c r="B183" t="s">
-        <v>9</v>
-      </c>
-      <c r="C183" t="s">
-        <v>10</v>
-      </c>
-      <c r="D183" t="s">
-        <v>27</v>
-      </c>
-      <c r="E183">
-        <v>764</v>
-      </c>
-      <c r="F183">
-        <v>4</v>
-      </c>
-      <c r="H183" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="184" spans="1:8">
-      <c r="A184" t="s">
-        <v>8</v>
-      </c>
-      <c r="B184" t="s">
-        <v>9</v>
-      </c>
-      <c r="C184" t="s">
-        <v>10</v>
-      </c>
-      <c r="D184" t="s">
-        <v>25</v>
-      </c>
-      <c r="E184">
-        <v>3962</v>
-      </c>
-      <c r="F184">
-        <v>4</v>
-      </c>
-      <c r="H184" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="185" spans="1:8">
-      <c r="A185" t="s">
-        <v>8</v>
-      </c>
-      <c r="B185" t="s">
-        <v>9</v>
-      </c>
-      <c r="C185" t="s">
-        <v>10</v>
-      </c>
-      <c r="D185" t="s">
-        <v>28</v>
-      </c>
-      <c r="E185">
-        <v>764</v>
-      </c>
-      <c r="F185">
-        <v>4</v>
-      </c>
-      <c r="H185" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="186" spans="1:8">
-      <c r="A186" t="s">
-        <v>8</v>
-      </c>
-      <c r="B186" t="s">
-        <v>9</v>
-      </c>
-      <c r="C186" t="s">
-        <v>10</v>
-      </c>
-      <c r="D186" t="s">
-        <v>26</v>
-      </c>
-      <c r="E186">
-        <v>3962</v>
-      </c>
-      <c r="F186">
-        <v>4</v>
-      </c>
-      <c r="H186" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>